<commit_message>
Add data for 2026-07-20
</commit_message>
<xml_diff>
--- a/output/cta-violent-crime-full-year.xlsx
+++ b/output/cta-violent-crime-full-year.xlsx
@@ -9,14 +9,14 @@
   <sheets>
     <sheet name="Citywide Totals" sheetId="1" r:id="rId1"/>
     <sheet name="By Neighborhood" sheetId="2" r:id="rId2"/>
-    <sheet name="Douglas" sheetId="3" r:id="rId3"/>
-    <sheet name="Avondale" sheetId="4" r:id="rId4"/>
-    <sheet name="Grand Crossing" sheetId="5" r:id="rId5"/>
-    <sheet name="Little Italy, UIC" sheetId="6" r:id="rId6"/>
-    <sheet name="Englewood" sheetId="7" r:id="rId7"/>
-    <sheet name="O'Hare" sheetId="8" r:id="rId8"/>
-    <sheet name="Austin" sheetId="9" r:id="rId9"/>
-    <sheet name="Loop" sheetId="10" r:id="rId10"/>
+    <sheet name="Austin" sheetId="3" r:id="rId3"/>
+    <sheet name="Loop" sheetId="4" r:id="rId4"/>
+    <sheet name="Little Italy, UIC" sheetId="5" r:id="rId5"/>
+    <sheet name="Douglas" sheetId="6" r:id="rId6"/>
+    <sheet name="Avondale" sheetId="7" r:id="rId7"/>
+    <sheet name="Grand Crossing" sheetId="8" r:id="rId8"/>
+    <sheet name="Englewood" sheetId="9" r:id="rId9"/>
+    <sheet name="O'Hare" sheetId="10" r:id="rId10"/>
     <sheet name="United Center" sheetId="11" r:id="rId11"/>
     <sheet name="Humboldt Park" sheetId="12" r:id="rId12"/>
     <sheet name="West Loop" sheetId="13" r:id="rId13"/>
@@ -930,7 +930,7 @@
         <v>262</v>
       </c>
       <c r="M3">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -1050,7 +1050,7 @@
         <v>467</v>
       </c>
       <c r="M6">
-        <v>150</v>
+        <v>152</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -1091,7 +1091,7 @@
         <v>893</v>
       </c>
       <c r="M7">
-        <v>367</v>
+        <v>370</v>
       </c>
     </row>
   </sheetData>
@@ -1101,7 +1101,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23.7109375" customWidth="1"/>
@@ -1116,10 +1116,9 @@
     <col min="10" max="10" width="4.7109375" customWidth="1"/>
     <col min="11" max="11" width="4.7109375" customWidth="1"/>
     <col min="12" max="12" width="4.7109375" customWidth="1"/>
-    <col min="13" max="13" width="4.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1139,244 +1138,163 @@
         <v>2019</v>
       </c>
       <c r="G1" s="1">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="H1" s="1">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="I1" s="1">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="J1" s="1">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="K1" s="1">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L1" s="1">
-        <v>2025</v>
-      </c>
-      <c r="M1" s="1">
         <v>2026</v>
       </c>
     </row>
-    <row r="2" spans="1:13">
+    <row r="2" spans="1:12">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B2">
-        <v>6</v>
-      </c>
-      <c r="C2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D2">
-        <v>12</v>
-      </c>
-      <c r="E2">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F2">
-        <v>8</v>
-      </c>
-      <c r="G2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H2">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="I2">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="J2">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="K2">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="L2">
-        <v>15</v>
-      </c>
-      <c r="M2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B3">
-        <v>13</v>
-      </c>
       <c r="C3">
-        <v>13</v>
-      </c>
-      <c r="D3">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="E3">
-        <v>18</v>
-      </c>
-      <c r="F3">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="G3">
-        <v>26</v>
+        <v>2</v>
       </c>
       <c r="H3">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="I3">
-        <v>32</v>
+        <v>1</v>
       </c>
       <c r="J3">
-        <v>40</v>
+        <v>2</v>
       </c>
       <c r="K3">
-        <v>26</v>
+        <v>2</v>
       </c>
       <c r="L3">
-        <v>34</v>
-      </c>
-      <c r="M3">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
       <c r="C4">
-        <v>2</v>
-      </c>
-      <c r="D4">
-        <v>1</v>
-      </c>
-      <c r="E4">
-        <v>2</v>
-      </c>
-      <c r="F4">
         <v>1</v>
       </c>
       <c r="H4">
-        <v>2</v>
-      </c>
-      <c r="I4">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J4">
-        <v>3</v>
-      </c>
-      <c r="K4">
-        <v>2</v>
-      </c>
-      <c r="L4">
-        <v>5</v>
-      </c>
-      <c r="M4">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12">
       <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G5">
-        <v>1</v>
-      </c>
-      <c r="H5">
-        <v>2</v>
-      </c>
-      <c r="J5">
-        <v>2</v>
-      </c>
-      <c r="L5">
-        <v>2</v>
-      </c>
-      <c r="M5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
+      <c r="K5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12">
       <c r="A6" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B6">
-        <v>30</v>
-      </c>
-      <c r="C6">
-        <v>44</v>
-      </c>
-      <c r="D6">
-        <v>49</v>
-      </c>
-      <c r="E6">
-        <v>67</v>
+        <v>1</v>
       </c>
       <c r="F6">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="G6">
-        <v>57</v>
+        <v>1</v>
       </c>
       <c r="H6">
-        <v>80</v>
-      </c>
-      <c r="I6">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="J6">
-        <v>64</v>
-      </c>
-      <c r="K6">
-        <v>48</v>
+        <v>1</v>
       </c>
       <c r="L6">
-        <v>44</v>
-      </c>
-      <c r="M6">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12">
       <c r="A7" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B7">
-        <v>49</v>
+        <v>2</v>
       </c>
       <c r="C7">
-        <v>62</v>
+        <v>2</v>
       </c>
       <c r="D7">
-        <v>79</v>
+        <v>2</v>
       </c>
       <c r="E7">
-        <v>92</v>
+        <v>1</v>
       </c>
       <c r="F7">
-        <v>92</v>
+        <v>6</v>
       </c>
       <c r="G7">
-        <v>88</v>
+        <v>3</v>
       </c>
       <c r="H7">
-        <v>120</v>
+        <v>7</v>
       </c>
       <c r="I7">
-        <v>130</v>
+        <v>3</v>
       </c>
       <c r="J7">
-        <v>131</v>
+        <v>5</v>
       </c>
       <c r="K7">
-        <v>91</v>
+        <v>9</v>
       </c>
       <c r="L7">
-        <v>100</v>
-      </c>
-      <c r="M7">
-        <v>35</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -3858,7 +3776,7 @@
         <v>33</v>
       </c>
       <c r="M8">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -5229,7 +5147,7 @@
         <v>22</v>
       </c>
       <c r="M50">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="51" spans="1:13">
@@ -5352,7 +5270,7 @@
         <v>100</v>
       </c>
       <c r="M53">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="54" spans="1:13">
@@ -6915,7 +6833,7 @@
         <v>893</v>
       </c>
       <c r="M98">
-        <v>367</v>
+        <v>370</v>
       </c>
     </row>
   </sheetData>
@@ -8986,23 +8904,41 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="B2">
+        <v>4</v>
+      </c>
       <c r="C2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D2">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="E2">
+        <v>5</v>
+      </c>
+      <c r="F2">
+        <v>9</v>
+      </c>
+      <c r="G2">
+        <v>3</v>
       </c>
       <c r="H2">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J2">
-        <v>2</v>
+        <v>8</v>
+      </c>
+      <c r="K2">
+        <v>7</v>
       </c>
       <c r="L2">
-        <v>1</v>
+        <v>5</v>
+      </c>
+      <c r="M2">
+        <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -9010,35 +8946,62 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>1</v>
+        <v>4</v>
+      </c>
+      <c r="C3">
+        <v>5</v>
       </c>
       <c r="D3">
-        <v>2</v>
+        <v>6</v>
+      </c>
+      <c r="E3">
+        <v>7</v>
       </c>
       <c r="F3">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G3">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="H3">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="I3">
-        <v>2</v>
+        <v>6</v>
+      </c>
+      <c r="J3">
+        <v>10</v>
       </c>
       <c r="K3">
-        <v>2</v>
+        <v>12</v>
+      </c>
+      <c r="L3">
+        <v>14</v>
       </c>
       <c r="M3">
-        <v>2</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4">
+        <v>1</v>
+      </c>
       <c r="J4">
+        <v>3</v>
+      </c>
+      <c r="K4">
+        <v>2</v>
+      </c>
+      <c r="M4">
         <v>1</v>
       </c>
     </row>
@@ -9055,37 +9018,40 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>7</v>
+        <v>23</v>
       </c>
       <c r="C6">
-        <v>5</v>
+        <v>31</v>
       </c>
       <c r="D6">
-        <v>5</v>
+        <v>22</v>
       </c>
       <c r="E6">
-        <v>5</v>
+        <v>44</v>
       </c>
       <c r="F6">
-        <v>5</v>
+        <v>38</v>
       </c>
       <c r="G6">
-        <v>1</v>
+        <v>24</v>
       </c>
       <c r="H6">
-        <v>5</v>
+        <v>50</v>
       </c>
       <c r="I6">
-        <v>4</v>
+        <v>34</v>
       </c>
       <c r="J6">
-        <v>1</v>
+        <v>26</v>
       </c>
       <c r="K6">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="L6">
-        <v>6</v>
+        <v>14</v>
+      </c>
+      <c r="M6">
+        <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -9093,40 +9059,40 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="C7">
-        <v>7</v>
+        <v>40</v>
       </c>
       <c r="D7">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="E7">
-        <v>5</v>
+        <v>57</v>
       </c>
       <c r="F7">
-        <v>8</v>
+        <v>53</v>
       </c>
       <c r="G7">
-        <v>2</v>
+        <v>34</v>
       </c>
       <c r="H7">
-        <v>8</v>
+        <v>63</v>
       </c>
       <c r="I7">
-        <v>7</v>
+        <v>44</v>
       </c>
       <c r="J7">
-        <v>4</v>
+        <v>47</v>
       </c>
       <c r="K7">
-        <v>7</v>
+        <v>46</v>
       </c>
       <c r="L7">
-        <v>7</v>
+        <v>33</v>
       </c>
       <c r="M7">
-        <v>2</v>
+        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -10960,7 +10926,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23.7109375" customWidth="1"/>
@@ -11024,28 +10990,37 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D2">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="E2">
-        <v>2</v>
+        <v>5</v>
+      </c>
+      <c r="F2">
+        <v>8</v>
+      </c>
+      <c r="G2">
+        <v>4</v>
       </c>
       <c r="H2">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="I2">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="J2">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="K2">
-        <v>2</v>
+        <v>15</v>
+      </c>
+      <c r="L2">
+        <v>15</v>
       </c>
       <c r="M2">
         <v>2</v>
@@ -11055,113 +11030,178 @@
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
+      <c r="B3">
+        <v>13</v>
+      </c>
+      <c r="C3">
+        <v>13</v>
+      </c>
+      <c r="D3">
+        <v>17</v>
+      </c>
       <c r="E3">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="F3">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="G3">
-        <v>1</v>
+        <v>26</v>
+      </c>
+      <c r="H3">
+        <v>23</v>
+      </c>
+      <c r="I3">
+        <v>32</v>
       </c>
       <c r="J3">
-        <v>2</v>
+        <v>40</v>
+      </c>
+      <c r="K3">
+        <v>26</v>
       </c>
       <c r="L3">
-        <v>2</v>
+        <v>34</v>
       </c>
       <c r="M3">
-        <v>3</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B4">
-        <v>1</v>
+      <c r="C4">
+        <v>2</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4">
+        <v>2</v>
+      </c>
+      <c r="F4">
+        <v>1</v>
+      </c>
+      <c r="H4">
+        <v>2</v>
+      </c>
+      <c r="I4">
+        <v>4</v>
+      </c>
+      <c r="J4">
+        <v>3</v>
       </c>
       <c r="K4">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="L4">
+        <v>5</v>
+      </c>
+      <c r="M4">
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5">
-        <v>2</v>
-      </c>
-      <c r="C5">
-        <v>1</v>
-      </c>
-      <c r="D5">
-        <v>3</v>
-      </c>
-      <c r="E5">
-        <v>1</v>
-      </c>
-      <c r="F5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G5">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H5">
-        <v>5</v>
-      </c>
-      <c r="I5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J5">
-        <v>6</v>
-      </c>
-      <c r="K5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L5">
-        <v>3</v>
+        <v>2</v>
+      </c>
+      <c r="M5">
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B6">
-        <v>4</v>
+        <v>30</v>
       </c>
       <c r="C6">
-        <v>2</v>
+        <v>44</v>
       </c>
       <c r="D6">
-        <v>4</v>
+        <v>49</v>
       </c>
       <c r="E6">
-        <v>5</v>
+        <v>67</v>
       </c>
       <c r="F6">
-        <v>5</v>
+        <v>69</v>
       </c>
       <c r="G6">
-        <v>5</v>
+        <v>57</v>
       </c>
       <c r="H6">
-        <v>6</v>
+        <v>80</v>
       </c>
       <c r="I6">
-        <v>5</v>
+        <v>80</v>
       </c>
       <c r="J6">
-        <v>9</v>
+        <v>64</v>
       </c>
       <c r="K6">
-        <v>6</v>
+        <v>48</v>
       </c>
       <c r="L6">
-        <v>5</v>
+        <v>44</v>
       </c>
       <c r="M6">
-        <v>5</v>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>49</v>
+      </c>
+      <c r="C7">
+        <v>62</v>
+      </c>
+      <c r="D7">
+        <v>79</v>
+      </c>
+      <c r="E7">
+        <v>92</v>
+      </c>
+      <c r="F7">
+        <v>92</v>
+      </c>
+      <c r="G7">
+        <v>88</v>
+      </c>
+      <c r="H7">
+        <v>120</v>
+      </c>
+      <c r="I7">
+        <v>130</v>
+      </c>
+      <c r="J7">
+        <v>131</v>
+      </c>
+      <c r="K7">
+        <v>91</v>
+      </c>
+      <c r="L7">
+        <v>100</v>
+      </c>
+      <c r="M7">
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -13077,7 +13117,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23.7109375" customWidth="1"/>
@@ -13140,41 +13180,32 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2">
-        <v>5</v>
-      </c>
       <c r="C2">
         <v>3</v>
       </c>
       <c r="D2">
-        <v>7</v>
-      </c>
-      <c r="E2">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F2">
-        <v>5</v>
-      </c>
-      <c r="G2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H2">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I2">
         <v>4</v>
       </c>
       <c r="J2">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="K2">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M2">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -13182,54 +13213,54 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>3</v>
-      </c>
-      <c r="C3">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D3">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="E3">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="F3">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="G3">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="H3">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="I3">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="J3">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="K3">
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="L3">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="M3">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E4">
-        <v>1</v>
-      </c>
-      <c r="F4">
-        <v>2</v>
-      </c>
-      <c r="J4">
-        <v>2</v>
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="H4">
+        <v>2</v>
+      </c>
+      <c r="K4">
+        <v>3</v>
+      </c>
+      <c r="L4">
+        <v>1</v>
       </c>
       <c r="M4">
         <v>1</v>
@@ -13237,101 +13268,84 @@
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="B5">
+        <v>5</v>
+      </c>
+      <c r="C5">
+        <v>7</v>
+      </c>
+      <c r="D5">
+        <v>11</v>
       </c>
       <c r="E5">
-        <v>1</v>
+        <v>21</v>
+      </c>
+      <c r="F5">
+        <v>25</v>
+      </c>
+      <c r="G5">
+        <v>15</v>
+      </c>
+      <c r="H5">
+        <v>10</v>
       </c>
       <c r="I5">
-        <v>1</v>
+        <v>9</v>
+      </c>
+      <c r="J5">
+        <v>11</v>
       </c>
       <c r="K5">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="L5">
-        <v>1</v>
+        <v>11</v>
+      </c>
+      <c r="M5">
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B6">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="C6">
-        <v>37</v>
+        <v>10</v>
       </c>
       <c r="D6">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="E6">
+        <v>23</v>
+      </c>
+      <c r="F6">
+        <v>28</v>
+      </c>
+      <c r="G6">
+        <v>16</v>
+      </c>
+      <c r="H6">
+        <v>14</v>
+      </c>
+      <c r="I6">
+        <v>17</v>
+      </c>
+      <c r="J6">
+        <v>16</v>
+      </c>
+      <c r="K6">
+        <v>31</v>
+      </c>
+      <c r="L6">
         <v>22</v>
-      </c>
-      <c r="F6">
-        <v>27</v>
-      </c>
-      <c r="G6">
-        <v>15</v>
-      </c>
-      <c r="H6">
-        <v>25</v>
-      </c>
-      <c r="I6">
-        <v>21</v>
-      </c>
-      <c r="J6">
-        <v>26</v>
-      </c>
-      <c r="K6">
-        <v>49</v>
-      </c>
-      <c r="L6">
-        <v>44</v>
       </c>
       <c r="M6">
         <v>10</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
-      <c r="A7" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B7">
-        <v>32</v>
-      </c>
-      <c r="C7">
-        <v>42</v>
-      </c>
-      <c r="D7">
-        <v>36</v>
-      </c>
-      <c r="E7">
-        <v>38</v>
-      </c>
-      <c r="F7">
-        <v>53</v>
-      </c>
-      <c r="G7">
-        <v>28</v>
-      </c>
-      <c r="H7">
-        <v>39</v>
-      </c>
-      <c r="I7">
-        <v>39</v>
-      </c>
-      <c r="J7">
-        <v>47</v>
-      </c>
-      <c r="K7">
-        <v>74</v>
-      </c>
-      <c r="L7">
-        <v>63</v>
-      </c>
-      <c r="M7">
-        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -15273,7 +15287,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23.7109375" customWidth="1"/>
@@ -15337,31 +15351,22 @@
         <v>1</v>
       </c>
       <c r="C2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D2">
         <v>1</v>
       </c>
-      <c r="F2">
-        <v>2</v>
-      </c>
       <c r="H2">
         <v>1</v>
       </c>
       <c r="I2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J2">
-        <v>1</v>
-      </c>
-      <c r="K2">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L2">
-        <v>4</v>
-      </c>
-      <c r="M2">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -15369,136 +15374,123 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D3">
         <v>2</v>
       </c>
-      <c r="E3">
-        <v>2</v>
-      </c>
       <c r="F3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G3">
         <v>1</v>
       </c>
       <c r="H3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I3">
-        <v>4</v>
-      </c>
-      <c r="J3">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K3">
-        <v>5</v>
-      </c>
-      <c r="L3">
-        <v>6</v>
+        <v>2</v>
+      </c>
+      <c r="M3">
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B4">
-        <v>1</v>
-      </c>
-      <c r="H4">
-        <v>2</v>
-      </c>
-      <c r="K4">
-        <v>3</v>
-      </c>
-      <c r="L4">
-        <v>1</v>
-      </c>
-      <c r="M4">
+      <c r="J4">
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5">
-        <v>5</v>
-      </c>
-      <c r="C5">
-        <v>7</v>
-      </c>
-      <c r="D5">
-        <v>11</v>
-      </c>
-      <c r="E5">
-        <v>21</v>
-      </c>
-      <c r="F5">
-        <v>25</v>
-      </c>
-      <c r="G5">
-        <v>15</v>
-      </c>
-      <c r="H5">
-        <v>10</v>
-      </c>
-      <c r="I5">
-        <v>9</v>
-      </c>
-      <c r="J5">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="K5">
-        <v>18</v>
-      </c>
-      <c r="L5">
-        <v>11</v>
-      </c>
-      <c r="M5">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B6">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C6">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D6">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="E6">
-        <v>23</v>
+        <v>5</v>
       </c>
       <c r="F6">
-        <v>28</v>
+        <v>5</v>
       </c>
       <c r="G6">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="H6">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="I6">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="J6">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="K6">
-        <v>31</v>
+        <v>4</v>
       </c>
       <c r="L6">
-        <v>22</v>
-      </c>
-      <c r="M6">
-        <v>9</v>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>8</v>
+      </c>
+      <c r="C7">
+        <v>7</v>
+      </c>
+      <c r="D7">
+        <v>8</v>
+      </c>
+      <c r="E7">
+        <v>5</v>
+      </c>
+      <c r="F7">
+        <v>8</v>
+      </c>
+      <c r="G7">
+        <v>2</v>
+      </c>
+      <c r="H7">
+        <v>8</v>
+      </c>
+      <c r="I7">
+        <v>7</v>
+      </c>
+      <c r="J7">
+        <v>4</v>
+      </c>
+      <c r="K7">
+        <v>7</v>
+      </c>
+      <c r="L7">
+        <v>7</v>
+      </c>
+      <c r="M7">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -17253,7 +17245,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23.7109375" customWidth="1"/>
@@ -17316,35 +17308,29 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
       <c r="C2">
         <v>1</v>
       </c>
       <c r="D2">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E2">
-        <v>1</v>
-      </c>
-      <c r="F2">
-        <v>9</v>
-      </c>
-      <c r="G2">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="H2">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="I2">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="J2">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="K2">
-        <v>3</v>
-      </c>
-      <c r="L2">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="M2">
         <v>2</v>
@@ -17354,41 +17340,23 @@
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B3">
-        <v>5</v>
-      </c>
-      <c r="C3">
-        <v>5</v>
-      </c>
-      <c r="D3">
-        <v>18</v>
-      </c>
       <c r="E3">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="F3">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="G3">
-        <v>11</v>
-      </c>
-      <c r="H3">
-        <v>7</v>
-      </c>
-      <c r="I3">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="J3">
-        <v>12</v>
-      </c>
-      <c r="K3">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="L3">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="M3">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -17398,116 +17366,87 @@
       <c r="B4">
         <v>1</v>
       </c>
-      <c r="D4">
-        <v>1</v>
-      </c>
-      <c r="H4">
-        <v>2</v>
-      </c>
-      <c r="J4">
-        <v>1</v>
-      </c>
       <c r="K4">
         <v>1</v>
-      </c>
-      <c r="L4">
-        <v>1</v>
-      </c>
-      <c r="M4">
-        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5">
+        <v>3</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+      <c r="F5">
+        <v>3</v>
+      </c>
+      <c r="G5">
         <v>4</v>
       </c>
       <c r="H5">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I5">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="J5">
+        <v>6</v>
+      </c>
+      <c r="K5">
+        <v>3</v>
+      </c>
+      <c r="L5">
+        <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B6">
-        <v>34</v>
+        <v>4</v>
       </c>
       <c r="C6">
-        <v>45</v>
+        <v>2</v>
       </c>
       <c r="D6">
-        <v>25</v>
+        <v>4</v>
       </c>
       <c r="E6">
-        <v>22</v>
+        <v>5</v>
       </c>
       <c r="F6">
-        <v>42</v>
+        <v>5</v>
       </c>
       <c r="G6">
-        <v>32</v>
+        <v>5</v>
       </c>
       <c r="H6">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="I6">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="J6">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="K6">
-        <v>44</v>
+        <v>6</v>
       </c>
       <c r="L6">
-        <v>44</v>
+        <v>5</v>
       </c>
       <c r="M6">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
-      <c r="A7" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B7">
-        <v>40</v>
-      </c>
-      <c r="C7">
-        <v>51</v>
-      </c>
-      <c r="D7">
-        <v>50</v>
-      </c>
-      <c r="E7">
-        <v>33</v>
-      </c>
-      <c r="F7">
-        <v>63</v>
-      </c>
-      <c r="G7">
-        <v>50</v>
-      </c>
-      <c r="H7">
-        <v>47</v>
-      </c>
-      <c r="I7">
-        <v>45</v>
-      </c>
-      <c r="J7">
-        <v>37</v>
-      </c>
-      <c r="K7">
-        <v>68</v>
-      </c>
-      <c r="L7">
-        <v>71</v>
-      </c>
-      <c r="M7">
-        <v>22</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -19033,7 +18972,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23.7109375" customWidth="1"/>
@@ -19048,9 +18987,10 @@
     <col min="10" max="10" width="4.7109375" customWidth="1"/>
     <col min="11" max="11" width="4.7109375" customWidth="1"/>
     <col min="12" max="12" width="4.7109375" customWidth="1"/>
+    <col min="13" max="13" width="4.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12">
+    <row r="1" spans="1:13">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -19070,163 +19010,223 @@
         <v>2019</v>
       </c>
       <c r="G1" s="1">
+        <v>2020</v>
+      </c>
+      <c r="H1" s="1">
         <v>2021</v>
       </c>
-      <c r="H1" s="1">
+      <c r="I1" s="1">
         <v>2022</v>
       </c>
-      <c r="I1" s="1">
+      <c r="J1" s="1">
         <v>2023</v>
       </c>
-      <c r="J1" s="1">
+      <c r="K1" s="1">
         <v>2024</v>
       </c>
-      <c r="K1" s="1">
+      <c r="L1" s="1">
         <v>2025</v>
       </c>
-      <c r="L1" s="1">
+      <c r="M1" s="1">
         <v>2026</v>
       </c>
     </row>
-    <row r="2" spans="1:12">
+    <row r="2" spans="1:13">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B2">
-        <v>1</v>
+        <v>5</v>
+      </c>
+      <c r="C2">
+        <v>3</v>
       </c>
       <c r="D2">
-        <v>2</v>
+        <v>7</v>
+      </c>
+      <c r="E2">
+        <v>5</v>
       </c>
       <c r="F2">
-        <v>2</v>
+        <v>5</v>
+      </c>
+      <c r="G2">
+        <v>4</v>
       </c>
       <c r="H2">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J2">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="K2">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12">
+        <v>5</v>
+      </c>
+      <c r="M2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
+      <c r="B3">
+        <v>3</v>
+      </c>
       <c r="C3">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="D3">
+        <v>8</v>
       </c>
       <c r="E3">
-        <v>1</v>
+        <v>9</v>
+      </c>
+      <c r="F3">
+        <v>19</v>
       </c>
       <c r="G3">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="H3">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="I3">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="J3">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="K3">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="L3">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12">
+        <v>13</v>
+      </c>
+      <c r="M3">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C4">
-        <v>1</v>
-      </c>
-      <c r="H4">
-        <v>1</v>
+      <c r="E4">
+        <v>1</v>
+      </c>
+      <c r="F4">
+        <v>2</v>
       </c>
       <c r="J4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12">
+        <v>2</v>
+      </c>
+      <c r="M4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+      <c r="I5">
+        <v>1</v>
+      </c>
       <c r="K5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12">
+        <v>1</v>
+      </c>
+      <c r="L5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B6">
-        <v>1</v>
+        <v>24</v>
+      </c>
+      <c r="C6">
+        <v>37</v>
+      </c>
+      <c r="D6">
+        <v>21</v>
+      </c>
+      <c r="E6">
+        <v>22</v>
       </c>
       <c r="F6">
-        <v>4</v>
+        <v>27</v>
       </c>
       <c r="G6">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="H6">
-        <v>2</v>
+        <v>25</v>
+      </c>
+      <c r="I6">
+        <v>21</v>
       </c>
       <c r="J6">
-        <v>1</v>
+        <v>26</v>
+      </c>
+      <c r="K6">
+        <v>49</v>
       </c>
       <c r="L6">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12">
+        <v>44</v>
+      </c>
+      <c r="M6">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
       <c r="A7" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B7">
-        <v>2</v>
+        <v>32</v>
       </c>
       <c r="C7">
-        <v>2</v>
+        <v>42</v>
       </c>
       <c r="D7">
-        <v>2</v>
+        <v>36</v>
       </c>
       <c r="E7">
-        <v>1</v>
+        <v>38</v>
       </c>
       <c r="F7">
-        <v>6</v>
+        <v>53</v>
       </c>
       <c r="G7">
-        <v>3</v>
+        <v>28</v>
       </c>
       <c r="H7">
-        <v>7</v>
+        <v>39</v>
       </c>
       <c r="I7">
-        <v>3</v>
+        <v>39</v>
       </c>
       <c r="J7">
-        <v>5</v>
+        <v>47</v>
       </c>
       <c r="K7">
-        <v>9</v>
+        <v>74</v>
       </c>
       <c r="L7">
-        <v>7</v>
+        <v>63</v>
+      </c>
+      <c r="M7">
+        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -20315,41 +20315,38 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2">
-        <v>4</v>
-      </c>
       <c r="C2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D2">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E2">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F2">
         <v>9</v>
       </c>
       <c r="G2">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="H2">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="I2">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="J2">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K2">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="L2">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M2">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -20357,40 +20354,40 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C3">
         <v>5</v>
       </c>
       <c r="D3">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="E3">
+        <v>10</v>
+      </c>
+      <c r="F3">
+        <v>12</v>
+      </c>
+      <c r="G3">
+        <v>11</v>
+      </c>
+      <c r="H3">
         <v>7</v>
       </c>
-      <c r="F3">
-        <v>6</v>
-      </c>
-      <c r="G3">
-        <v>7</v>
-      </c>
-      <c r="H3">
-        <v>8</v>
-      </c>
       <c r="I3">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="J3">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="K3">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="L3">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="M3">
-        <v>9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -20403,24 +20400,30 @@
       <c r="D4">
         <v>1</v>
       </c>
-      <c r="E4">
-        <v>1</v>
+      <c r="H4">
+        <v>2</v>
       </c>
       <c r="J4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K4">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="L4">
+        <v>1</v>
       </c>
       <c r="M4">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="K5">
+      <c r="H5">
+        <v>1</v>
+      </c>
+      <c r="I5">
         <v>1</v>
       </c>
     </row>
@@ -20429,40 +20432,40 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>23</v>
+        <v>34</v>
       </c>
       <c r="C6">
-        <v>31</v>
+        <v>45</v>
       </c>
       <c r="D6">
+        <v>25</v>
+      </c>
+      <c r="E6">
         <v>22</v>
       </c>
-      <c r="E6">
+      <c r="F6">
+        <v>42</v>
+      </c>
+      <c r="G6">
+        <v>32</v>
+      </c>
+      <c r="H6">
+        <v>26</v>
+      </c>
+      <c r="I6">
+        <v>21</v>
+      </c>
+      <c r="J6">
+        <v>15</v>
+      </c>
+      <c r="K6">
         <v>44</v>
       </c>
-      <c r="F6">
-        <v>38</v>
-      </c>
-      <c r="G6">
-        <v>24</v>
-      </c>
-      <c r="H6">
-        <v>50</v>
-      </c>
-      <c r="I6">
-        <v>34</v>
-      </c>
-      <c r="J6">
-        <v>26</v>
-      </c>
-      <c r="K6">
-        <v>24</v>
-      </c>
       <c r="L6">
+        <v>44</v>
+      </c>
+      <c r="M6">
         <v>14</v>
-      </c>
-      <c r="M6">
-        <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -20470,40 +20473,40 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="C7">
-        <v>40</v>
+        <v>51</v>
       </c>
       <c r="D7">
-        <v>32</v>
+        <v>50</v>
       </c>
       <c r="E7">
-        <v>57</v>
+        <v>33</v>
       </c>
       <c r="F7">
-        <v>53</v>
+        <v>63</v>
       </c>
       <c r="G7">
-        <v>34</v>
+        <v>50</v>
       </c>
       <c r="H7">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="I7">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="J7">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="K7">
-        <v>46</v>
+        <v>68</v>
       </c>
       <c r="L7">
-        <v>33</v>
+        <v>71</v>
       </c>
       <c r="M7">
-        <v>30</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add data for 2026-07-26
</commit_message>
<xml_diff>
--- a/output/cta-violent-crime-full-year.xlsx
+++ b/output/cta-violent-crime-full-year.xlsx
@@ -9,24 +9,24 @@
   <sheets>
     <sheet name="Citywide Totals" sheetId="1" r:id="rId1"/>
     <sheet name="By Neighborhood" sheetId="2" r:id="rId2"/>
-    <sheet name="Loop" sheetId="3" r:id="rId3"/>
-    <sheet name="Fuller Park" sheetId="4" r:id="rId4"/>
-    <sheet name="South Chicago" sheetId="5" r:id="rId5"/>
-    <sheet name="Armour Square" sheetId="6" r:id="rId6"/>
-    <sheet name="Austin" sheetId="7" r:id="rId7"/>
-    <sheet name="Little Italy, UIC" sheetId="8" r:id="rId8"/>
-    <sheet name="Douglas" sheetId="9" r:id="rId9"/>
-    <sheet name="Avondale" sheetId="10" r:id="rId10"/>
-    <sheet name="Grand Crossing" sheetId="11" r:id="rId11"/>
-    <sheet name="Englewood" sheetId="12" r:id="rId12"/>
-    <sheet name="O'Hare" sheetId="13" r:id="rId13"/>
-    <sheet name="United Center" sheetId="14" r:id="rId14"/>
-    <sheet name="Humboldt Park" sheetId="15" r:id="rId15"/>
-    <sheet name="West Loop" sheetId="16" r:id="rId16"/>
-    <sheet name="Garfield Park" sheetId="17" r:id="rId17"/>
-    <sheet name="Roseland" sheetId="18" r:id="rId18"/>
-    <sheet name="Washington Park" sheetId="19" r:id="rId19"/>
-    <sheet name="Chatham" sheetId="20" r:id="rId20"/>
+    <sheet name="Chatham" sheetId="3" r:id="rId3"/>
+    <sheet name="Loop" sheetId="4" r:id="rId4"/>
+    <sheet name="Fuller Park" sheetId="5" r:id="rId5"/>
+    <sheet name="South Chicago" sheetId="6" r:id="rId6"/>
+    <sheet name="Armour Square" sheetId="7" r:id="rId7"/>
+    <sheet name="Austin" sheetId="8" r:id="rId8"/>
+    <sheet name="Little Italy, UIC" sheetId="9" r:id="rId9"/>
+    <sheet name="Douglas" sheetId="10" r:id="rId10"/>
+    <sheet name="Avondale" sheetId="11" r:id="rId11"/>
+    <sheet name="Grand Crossing" sheetId="12" r:id="rId12"/>
+    <sheet name="Englewood" sheetId="13" r:id="rId13"/>
+    <sheet name="O'Hare" sheetId="14" r:id="rId14"/>
+    <sheet name="United Center" sheetId="15" r:id="rId15"/>
+    <sheet name="Humboldt Park" sheetId="16" r:id="rId16"/>
+    <sheet name="West Loop" sheetId="17" r:id="rId17"/>
+    <sheet name="Garfield Park" sheetId="18" r:id="rId18"/>
+    <sheet name="Roseland" sheetId="19" r:id="rId19"/>
+    <sheet name="Washington Park" sheetId="20" r:id="rId20"/>
     <sheet name="Uptown" sheetId="21" r:id="rId21"/>
     <sheet name="Lake View" sheetId="22" r:id="rId22"/>
     <sheet name="Grant Park" sheetId="23" r:id="rId23"/>
@@ -930,7 +930,7 @@
         <v>262</v>
       </c>
       <c r="M3">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -1091,7 +1091,7 @@
         <v>893</v>
       </c>
       <c r="M7">
-        <v>375</v>
+        <v>376</v>
       </c>
     </row>
   </sheetData>
@@ -1100,6 +1100,219 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:M7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="2" max="2" width="4.7109375" customWidth="1"/>
+    <col min="3" max="3" width="4.7109375" customWidth="1"/>
+    <col min="4" max="4" width="4.7109375" customWidth="1"/>
+    <col min="5" max="5" width="4.7109375" customWidth="1"/>
+    <col min="6" max="6" width="4.7109375" customWidth="1"/>
+    <col min="7" max="7" width="4.7109375" customWidth="1"/>
+    <col min="8" max="8" width="4.7109375" customWidth="1"/>
+    <col min="9" max="9" width="4.7109375" customWidth="1"/>
+    <col min="10" max="10" width="4.7109375" customWidth="1"/>
+    <col min="11" max="11" width="4.7109375" customWidth="1"/>
+    <col min="12" max="12" width="4.7109375" customWidth="1"/>
+    <col min="13" max="13" width="4.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1">
+        <v>2015</v>
+      </c>
+      <c r="C1" s="1">
+        <v>2016</v>
+      </c>
+      <c r="D1" s="1">
+        <v>2017</v>
+      </c>
+      <c r="E1" s="1">
+        <v>2018</v>
+      </c>
+      <c r="F1" s="1">
+        <v>2019</v>
+      </c>
+      <c r="G1" s="1">
+        <v>2020</v>
+      </c>
+      <c r="H1" s="1">
+        <v>2021</v>
+      </c>
+      <c r="I1" s="1">
+        <v>2022</v>
+      </c>
+      <c r="J1" s="1">
+        <v>2023</v>
+      </c>
+      <c r="K1" s="1">
+        <v>2024</v>
+      </c>
+      <c r="L1" s="1">
+        <v>2025</v>
+      </c>
+      <c r="M1" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>2</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="H2">
+        <v>1</v>
+      </c>
+      <c r="I2">
+        <v>1</v>
+      </c>
+      <c r="J2">
+        <v>2</v>
+      </c>
+      <c r="L2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>2</v>
+      </c>
+      <c r="F3">
+        <v>3</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="H3">
+        <v>2</v>
+      </c>
+      <c r="I3">
+        <v>2</v>
+      </c>
+      <c r="K3">
+        <v>2</v>
+      </c>
+      <c r="M3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="J4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="K5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>7</v>
+      </c>
+      <c r="C6">
+        <v>5</v>
+      </c>
+      <c r="D6">
+        <v>5</v>
+      </c>
+      <c r="E6">
+        <v>5</v>
+      </c>
+      <c r="F6">
+        <v>5</v>
+      </c>
+      <c r="G6">
+        <v>1</v>
+      </c>
+      <c r="H6">
+        <v>5</v>
+      </c>
+      <c r="I6">
+        <v>4</v>
+      </c>
+      <c r="J6">
+        <v>1</v>
+      </c>
+      <c r="K6">
+        <v>4</v>
+      </c>
+      <c r="L6">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>8</v>
+      </c>
+      <c r="C7">
+        <v>7</v>
+      </c>
+      <c r="D7">
+        <v>8</v>
+      </c>
+      <c r="E7">
+        <v>5</v>
+      </c>
+      <c r="F7">
+        <v>8</v>
+      </c>
+      <c r="G7">
+        <v>2</v>
+      </c>
+      <c r="H7">
+        <v>8</v>
+      </c>
+      <c r="I7">
+        <v>7</v>
+      </c>
+      <c r="J7">
+        <v>4</v>
+      </c>
+      <c r="K7">
+        <v>7</v>
+      </c>
+      <c r="L7">
+        <v>7</v>
+      </c>
+      <c r="M7">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1303,270 +1516,6 @@
       </c>
       <c r="M6">
         <v>5</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M7"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
-    <col min="2" max="2" width="4.7109375" customWidth="1"/>
-    <col min="3" max="3" width="4.7109375" customWidth="1"/>
-    <col min="4" max="4" width="4.7109375" customWidth="1"/>
-    <col min="5" max="5" width="4.7109375" customWidth="1"/>
-    <col min="6" max="6" width="4.7109375" customWidth="1"/>
-    <col min="7" max="7" width="4.7109375" customWidth="1"/>
-    <col min="8" max="8" width="4.7109375" customWidth="1"/>
-    <col min="9" max="9" width="4.7109375" customWidth="1"/>
-    <col min="10" max="10" width="4.7109375" customWidth="1"/>
-    <col min="11" max="11" width="4.7109375" customWidth="1"/>
-    <col min="12" max="12" width="4.7109375" customWidth="1"/>
-    <col min="13" max="13" width="4.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:13">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1">
-        <v>2015</v>
-      </c>
-      <c r="C1" s="1">
-        <v>2016</v>
-      </c>
-      <c r="D1" s="1">
-        <v>2017</v>
-      </c>
-      <c r="E1" s="1">
-        <v>2018</v>
-      </c>
-      <c r="F1" s="1">
-        <v>2019</v>
-      </c>
-      <c r="G1" s="1">
-        <v>2020</v>
-      </c>
-      <c r="H1" s="1">
-        <v>2021</v>
-      </c>
-      <c r="I1" s="1">
-        <v>2022</v>
-      </c>
-      <c r="J1" s="1">
-        <v>2023</v>
-      </c>
-      <c r="K1" s="1">
-        <v>2024</v>
-      </c>
-      <c r="L1" s="1">
-        <v>2025</v>
-      </c>
-      <c r="M1" s="1">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2">
-        <v>5</v>
-      </c>
-      <c r="C2">
-        <v>3</v>
-      </c>
-      <c r="D2">
-        <v>7</v>
-      </c>
-      <c r="E2">
-        <v>5</v>
-      </c>
-      <c r="F2">
-        <v>5</v>
-      </c>
-      <c r="G2">
-        <v>4</v>
-      </c>
-      <c r="H2">
-        <v>6</v>
-      </c>
-      <c r="I2">
-        <v>4</v>
-      </c>
-      <c r="J2">
-        <v>7</v>
-      </c>
-      <c r="K2">
-        <v>7</v>
-      </c>
-      <c r="L2">
-        <v>5</v>
-      </c>
-      <c r="M2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
-      <c r="A3" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3">
-        <v>3</v>
-      </c>
-      <c r="C3">
-        <v>2</v>
-      </c>
-      <c r="D3">
-        <v>8</v>
-      </c>
-      <c r="E3">
-        <v>9</v>
-      </c>
-      <c r="F3">
-        <v>19</v>
-      </c>
-      <c r="G3">
-        <v>9</v>
-      </c>
-      <c r="H3">
-        <v>8</v>
-      </c>
-      <c r="I3">
-        <v>13</v>
-      </c>
-      <c r="J3">
-        <v>12</v>
-      </c>
-      <c r="K3">
-        <v>17</v>
-      </c>
-      <c r="L3">
-        <v>13</v>
-      </c>
-      <c r="M3">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
-      <c r="A4" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E4">
-        <v>1</v>
-      </c>
-      <c r="F4">
-        <v>2</v>
-      </c>
-      <c r="J4">
-        <v>2</v>
-      </c>
-      <c r="M4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
-      <c r="A5" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="E5">
-        <v>1</v>
-      </c>
-      <c r="I5">
-        <v>1</v>
-      </c>
-      <c r="K5">
-        <v>1</v>
-      </c>
-      <c r="L5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
-      <c r="A6" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B6">
-        <v>24</v>
-      </c>
-      <c r="C6">
-        <v>37</v>
-      </c>
-      <c r="D6">
-        <v>21</v>
-      </c>
-      <c r="E6">
-        <v>22</v>
-      </c>
-      <c r="F6">
-        <v>27</v>
-      </c>
-      <c r="G6">
-        <v>15</v>
-      </c>
-      <c r="H6">
-        <v>25</v>
-      </c>
-      <c r="I6">
-        <v>21</v>
-      </c>
-      <c r="J6">
-        <v>26</v>
-      </c>
-      <c r="K6">
-        <v>49</v>
-      </c>
-      <c r="L6">
-        <v>44</v>
-      </c>
-      <c r="M6">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
-      <c r="A7" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B7">
-        <v>32</v>
-      </c>
-      <c r="C7">
-        <v>42</v>
-      </c>
-      <c r="D7">
-        <v>36</v>
-      </c>
-      <c r="E7">
-        <v>38</v>
-      </c>
-      <c r="F7">
-        <v>53</v>
-      </c>
-      <c r="G7">
-        <v>28</v>
-      </c>
-      <c r="H7">
-        <v>39</v>
-      </c>
-      <c r="I7">
-        <v>39</v>
-      </c>
-      <c r="J7">
-        <v>47</v>
-      </c>
-      <c r="K7">
-        <v>74</v>
-      </c>
-      <c r="L7">
-        <v>63</v>
-      </c>
-      <c r="M7">
-        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -1639,38 +1588,41 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="B2">
+        <v>5</v>
+      </c>
       <c r="C2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D2">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E2">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F2">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="G2">
+        <v>4</v>
+      </c>
+      <c r="H2">
+        <v>6</v>
+      </c>
+      <c r="I2">
+        <v>4</v>
+      </c>
+      <c r="J2">
         <v>7</v>
       </c>
-      <c r="H2">
-        <v>11</v>
-      </c>
-      <c r="I2">
-        <v>10</v>
-      </c>
-      <c r="J2">
-        <v>9</v>
-      </c>
       <c r="K2">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="L2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M2">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -1678,25 +1630,25 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C3">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D3">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="E3">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F3">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="G3">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="H3">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I3">
         <v>13</v>
@@ -1705,49 +1657,46 @@
         <v>12</v>
       </c>
       <c r="K3">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="L3">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="M3">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B4">
-        <v>1</v>
-      </c>
-      <c r="D4">
-        <v>1</v>
-      </c>
-      <c r="H4">
+      <c r="E4">
+        <v>1</v>
+      </c>
+      <c r="F4">
         <v>2</v>
       </c>
       <c r="J4">
-        <v>1</v>
-      </c>
-      <c r="K4">
-        <v>1</v>
-      </c>
-      <c r="L4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M4">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="H5">
+      <c r="E5">
         <v>1</v>
       </c>
       <c r="I5">
+        <v>1</v>
+      </c>
+      <c r="K5">
+        <v>1</v>
+      </c>
+      <c r="L5">
         <v>1</v>
       </c>
     </row>
@@ -1756,40 +1705,40 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="C6">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="D6">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="E6">
         <v>22</v>
       </c>
       <c r="F6">
-        <v>42</v>
+        <v>27</v>
       </c>
       <c r="G6">
-        <v>32</v>
+        <v>15</v>
       </c>
       <c r="H6">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="I6">
         <v>21</v>
       </c>
       <c r="J6">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="K6">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="L6">
         <v>44</v>
       </c>
       <c r="M6">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -1797,40 +1746,40 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="C7">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="D7">
-        <v>50</v>
+        <v>36</v>
       </c>
       <c r="E7">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="F7">
+        <v>53</v>
+      </c>
+      <c r="G7">
+        <v>28</v>
+      </c>
+      <c r="H7">
+        <v>39</v>
+      </c>
+      <c r="I7">
+        <v>39</v>
+      </c>
+      <c r="J7">
+        <v>47</v>
+      </c>
+      <c r="K7">
+        <v>74</v>
+      </c>
+      <c r="L7">
         <v>63</v>
       </c>
-      <c r="G7">
-        <v>50</v>
-      </c>
-      <c r="H7">
-        <v>47</v>
-      </c>
-      <c r="I7">
-        <v>45</v>
-      </c>
-      <c r="J7">
-        <v>37</v>
-      </c>
-      <c r="K7">
-        <v>68</v>
-      </c>
-      <c r="L7">
-        <v>71</v>
-      </c>
       <c r="M7">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -1839,6 +1788,270 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:M7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="2" max="2" width="4.7109375" customWidth="1"/>
+    <col min="3" max="3" width="4.7109375" customWidth="1"/>
+    <col min="4" max="4" width="4.7109375" customWidth="1"/>
+    <col min="5" max="5" width="4.7109375" customWidth="1"/>
+    <col min="6" max="6" width="4.7109375" customWidth="1"/>
+    <col min="7" max="7" width="4.7109375" customWidth="1"/>
+    <col min="8" max="8" width="4.7109375" customWidth="1"/>
+    <col min="9" max="9" width="4.7109375" customWidth="1"/>
+    <col min="10" max="10" width="4.7109375" customWidth="1"/>
+    <col min="11" max="11" width="4.7109375" customWidth="1"/>
+    <col min="12" max="12" width="4.7109375" customWidth="1"/>
+    <col min="13" max="13" width="4.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1">
+        <v>2015</v>
+      </c>
+      <c r="C1" s="1">
+        <v>2016</v>
+      </c>
+      <c r="D1" s="1">
+        <v>2017</v>
+      </c>
+      <c r="E1" s="1">
+        <v>2018</v>
+      </c>
+      <c r="F1" s="1">
+        <v>2019</v>
+      </c>
+      <c r="G1" s="1">
+        <v>2020</v>
+      </c>
+      <c r="H1" s="1">
+        <v>2021</v>
+      </c>
+      <c r="I1" s="1">
+        <v>2022</v>
+      </c>
+      <c r="J1" s="1">
+        <v>2023</v>
+      </c>
+      <c r="K1" s="1">
+        <v>2024</v>
+      </c>
+      <c r="L1" s="1">
+        <v>2025</v>
+      </c>
+      <c r="M1" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>6</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2">
+        <v>9</v>
+      </c>
+      <c r="G2">
+        <v>7</v>
+      </c>
+      <c r="H2">
+        <v>11</v>
+      </c>
+      <c r="I2">
+        <v>10</v>
+      </c>
+      <c r="J2">
+        <v>9</v>
+      </c>
+      <c r="K2">
+        <v>3</v>
+      </c>
+      <c r="L2">
+        <v>6</v>
+      </c>
+      <c r="M2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>5</v>
+      </c>
+      <c r="C3">
+        <v>5</v>
+      </c>
+      <c r="D3">
+        <v>18</v>
+      </c>
+      <c r="E3">
+        <v>10</v>
+      </c>
+      <c r="F3">
+        <v>12</v>
+      </c>
+      <c r="G3">
+        <v>11</v>
+      </c>
+      <c r="H3">
+        <v>7</v>
+      </c>
+      <c r="I3">
+        <v>13</v>
+      </c>
+      <c r="J3">
+        <v>12</v>
+      </c>
+      <c r="K3">
+        <v>20</v>
+      </c>
+      <c r="L3">
+        <v>20</v>
+      </c>
+      <c r="M3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="H4">
+        <v>2</v>
+      </c>
+      <c r="J4">
+        <v>1</v>
+      </c>
+      <c r="K4">
+        <v>1</v>
+      </c>
+      <c r="L4">
+        <v>1</v>
+      </c>
+      <c r="M4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="H5">
+        <v>1</v>
+      </c>
+      <c r="I5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>34</v>
+      </c>
+      <c r="C6">
+        <v>45</v>
+      </c>
+      <c r="D6">
+        <v>25</v>
+      </c>
+      <c r="E6">
+        <v>22</v>
+      </c>
+      <c r="F6">
+        <v>42</v>
+      </c>
+      <c r="G6">
+        <v>32</v>
+      </c>
+      <c r="H6">
+        <v>26</v>
+      </c>
+      <c r="I6">
+        <v>21</v>
+      </c>
+      <c r="J6">
+        <v>15</v>
+      </c>
+      <c r="K6">
+        <v>44</v>
+      </c>
+      <c r="L6">
+        <v>44</v>
+      </c>
+      <c r="M6">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>40</v>
+      </c>
+      <c r="C7">
+        <v>51</v>
+      </c>
+      <c r="D7">
+        <v>50</v>
+      </c>
+      <c r="E7">
+        <v>33</v>
+      </c>
+      <c r="F7">
+        <v>63</v>
+      </c>
+      <c r="G7">
+        <v>50</v>
+      </c>
+      <c r="H7">
+        <v>47</v>
+      </c>
+      <c r="I7">
+        <v>45</v>
+      </c>
+      <c r="J7">
+        <v>37</v>
+      </c>
+      <c r="K7">
+        <v>68</v>
+      </c>
+      <c r="L7">
+        <v>71</v>
+      </c>
+      <c r="M7">
+        <v>22</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:L7"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2041,7 +2254,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2264,7 +2477,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2492,243 +2705,6 @@
       </c>
       <c r="M6">
         <v>8</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M7"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
-    <col min="2" max="2" width="4.7109375" customWidth="1"/>
-    <col min="3" max="3" width="4.7109375" customWidth="1"/>
-    <col min="4" max="4" width="4.7109375" customWidth="1"/>
-    <col min="5" max="5" width="4.7109375" customWidth="1"/>
-    <col min="6" max="6" width="4.7109375" customWidth="1"/>
-    <col min="7" max="7" width="4.7109375" customWidth="1"/>
-    <col min="8" max="8" width="4.7109375" customWidth="1"/>
-    <col min="9" max="9" width="4.7109375" customWidth="1"/>
-    <col min="10" max="10" width="4.7109375" customWidth="1"/>
-    <col min="11" max="11" width="4.7109375" customWidth="1"/>
-    <col min="12" max="12" width="4.7109375" customWidth="1"/>
-    <col min="13" max="13" width="4.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:13">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1">
-        <v>2015</v>
-      </c>
-      <c r="C1" s="1">
-        <v>2016</v>
-      </c>
-      <c r="D1" s="1">
-        <v>2017</v>
-      </c>
-      <c r="E1" s="1">
-        <v>2018</v>
-      </c>
-      <c r="F1" s="1">
-        <v>2019</v>
-      </c>
-      <c r="G1" s="1">
-        <v>2020</v>
-      </c>
-      <c r="H1" s="1">
-        <v>2021</v>
-      </c>
-      <c r="I1" s="1">
-        <v>2022</v>
-      </c>
-      <c r="J1" s="1">
-        <v>2023</v>
-      </c>
-      <c r="K1" s="1">
-        <v>2024</v>
-      </c>
-      <c r="L1" s="1">
-        <v>2025</v>
-      </c>
-      <c r="M1" s="1">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
-      <c r="C2">
-        <v>2</v>
-      </c>
-      <c r="G2">
-        <v>2</v>
-      </c>
-      <c r="H2">
-        <v>4</v>
-      </c>
-      <c r="I2">
-        <v>3</v>
-      </c>
-      <c r="J2">
-        <v>2</v>
-      </c>
-      <c r="K2">
-        <v>2</v>
-      </c>
-      <c r="L2">
-        <v>1</v>
-      </c>
-      <c r="M2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
-      <c r="A3" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3">
-        <v>1</v>
-      </c>
-      <c r="D3">
-        <v>2</v>
-      </c>
-      <c r="E3">
-        <v>1</v>
-      </c>
-      <c r="F3">
-        <v>1</v>
-      </c>
-      <c r="G3">
-        <v>2</v>
-      </c>
-      <c r="H3">
-        <v>3</v>
-      </c>
-      <c r="I3">
-        <v>2</v>
-      </c>
-      <c r="J3">
-        <v>1</v>
-      </c>
-      <c r="K3">
-        <v>5</v>
-      </c>
-      <c r="L3">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
-      <c r="A4" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F4">
-        <v>1</v>
-      </c>
-      <c r="J4">
-        <v>1</v>
-      </c>
-      <c r="L4">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
-      <c r="A5" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="I5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
-      <c r="A6" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B6">
-        <v>5</v>
-      </c>
-      <c r="C6">
-        <v>1</v>
-      </c>
-      <c r="D6">
-        <v>6</v>
-      </c>
-      <c r="E6">
-        <v>8</v>
-      </c>
-      <c r="F6">
-        <v>10</v>
-      </c>
-      <c r="G6">
-        <v>8</v>
-      </c>
-      <c r="H6">
-        <v>9</v>
-      </c>
-      <c r="I6">
-        <v>7</v>
-      </c>
-      <c r="J6">
-        <v>4</v>
-      </c>
-      <c r="K6">
-        <v>7</v>
-      </c>
-      <c r="L6">
-        <v>5</v>
-      </c>
-      <c r="M6">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
-      <c r="A7" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B7">
-        <v>7</v>
-      </c>
-      <c r="C7">
-        <v>3</v>
-      </c>
-      <c r="D7">
-        <v>8</v>
-      </c>
-      <c r="E7">
-        <v>9</v>
-      </c>
-      <c r="F7">
-        <v>12</v>
-      </c>
-      <c r="G7">
-        <v>12</v>
-      </c>
-      <c r="H7">
-        <v>16</v>
-      </c>
-      <c r="I7">
-        <v>13</v>
-      </c>
-      <c r="J7">
-        <v>8</v>
-      </c>
-      <c r="K7">
-        <v>14</v>
-      </c>
-      <c r="L7">
-        <v>15</v>
-      </c>
-      <c r="M7">
-        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -2807,35 +2783,26 @@
       <c r="C2">
         <v>2</v>
       </c>
-      <c r="D2">
-        <v>7</v>
-      </c>
-      <c r="E2">
-        <v>8</v>
-      </c>
-      <c r="F2">
-        <v>5</v>
-      </c>
       <c r="G2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K2">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L2">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="M2">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -2845,64 +2812,46 @@
       <c r="B3">
         <v>1</v>
       </c>
-      <c r="C3">
-        <v>3</v>
-      </c>
       <c r="D3">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="E3">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F3">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G3">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="H3">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="I3">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="J3">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="K3">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="L3">
-        <v>8</v>
-      </c>
-      <c r="M3">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B4">
-        <v>2</v>
-      </c>
-      <c r="D4">
-        <v>1</v>
-      </c>
-      <c r="E4">
-        <v>1</v>
-      </c>
       <c r="F4">
         <v>1</v>
       </c>
-      <c r="H4">
-        <v>1</v>
-      </c>
-      <c r="I4">
-        <v>2</v>
-      </c>
-      <c r="M4">
-        <v>1</v>
+      <c r="J4">
+        <v>1</v>
+      </c>
+      <c r="L4">
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -2918,40 +2867,40 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="C6">
-        <v>35</v>
+        <v>1</v>
       </c>
       <c r="D6">
-        <v>34</v>
+        <v>6</v>
       </c>
       <c r="E6">
-        <v>56</v>
+        <v>8</v>
       </c>
       <c r="F6">
-        <v>54</v>
+        <v>10</v>
       </c>
       <c r="G6">
-        <v>37</v>
+        <v>8</v>
       </c>
       <c r="H6">
-        <v>39</v>
+        <v>9</v>
       </c>
       <c r="I6">
-        <v>32</v>
+        <v>7</v>
       </c>
       <c r="J6">
-        <v>34</v>
+        <v>4</v>
       </c>
       <c r="K6">
-        <v>27</v>
+        <v>7</v>
       </c>
       <c r="L6">
-        <v>31</v>
+        <v>5</v>
       </c>
       <c r="M6">
-        <v>11</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -2959,40 +2908,40 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>19</v>
+        <v>7</v>
       </c>
       <c r="C7">
-        <v>40</v>
+        <v>3</v>
       </c>
       <c r="D7">
-        <v>51</v>
+        <v>8</v>
       </c>
       <c r="E7">
-        <v>69</v>
+        <v>9</v>
       </c>
       <c r="F7">
-        <v>65</v>
+        <v>12</v>
       </c>
       <c r="G7">
-        <v>47</v>
+        <v>12</v>
       </c>
       <c r="H7">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="I7">
-        <v>49</v>
+        <v>13</v>
       </c>
       <c r="J7">
-        <v>51</v>
+        <v>8</v>
       </c>
       <c r="K7">
-        <v>48</v>
+        <v>14</v>
       </c>
       <c r="L7">
-        <v>44</v>
+        <v>15</v>
       </c>
       <c r="M7">
-        <v>25</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -3066,40 +3015,40 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D2">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E2">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="F2">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H2">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="I2">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K2">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L2">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M2">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -3107,25 +3056,25 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C3">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D3">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="E3">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F3">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="G3">
         <v>6</v>
       </c>
       <c r="H3">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="I3">
         <v>9</v>
@@ -3134,36 +3083,36 @@
         <v>14</v>
       </c>
       <c r="K3">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="L3">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="M3">
-        <v>2</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C4">
-        <v>1</v>
-      </c>
-      <c r="G4">
+      <c r="B4">
+        <v>2</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4">
+        <v>1</v>
+      </c>
+      <c r="F4">
+        <v>1</v>
+      </c>
+      <c r="H4">
         <v>1</v>
       </c>
       <c r="I4">
         <v>2</v>
-      </c>
-      <c r="J4">
-        <v>1</v>
-      </c>
-      <c r="K4">
-        <v>1</v>
-      </c>
-      <c r="L4">
-        <v>1</v>
       </c>
       <c r="M4">
         <v>1</v>
@@ -3173,7 +3122,7 @@
       <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D5">
+      <c r="I5">
         <v>1</v>
       </c>
     </row>
@@ -3182,40 +3131,40 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="C6">
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="D6">
+        <v>34</v>
+      </c>
+      <c r="E6">
+        <v>56</v>
+      </c>
+      <c r="F6">
+        <v>54</v>
+      </c>
+      <c r="G6">
+        <v>37</v>
+      </c>
+      <c r="H6">
+        <v>39</v>
+      </c>
+      <c r="I6">
+        <v>32</v>
+      </c>
+      <c r="J6">
+        <v>34</v>
+      </c>
+      <c r="K6">
+        <v>27</v>
+      </c>
+      <c r="L6">
+        <v>31</v>
+      </c>
+      <c r="M6">
         <v>11</v>
-      </c>
-      <c r="E6">
-        <v>14</v>
-      </c>
-      <c r="F6">
-        <v>12</v>
-      </c>
-      <c r="G6">
-        <v>14</v>
-      </c>
-      <c r="H6">
-        <v>19</v>
-      </c>
-      <c r="I6">
-        <v>29</v>
-      </c>
-      <c r="J6">
-        <v>19</v>
-      </c>
-      <c r="K6">
-        <v>20</v>
-      </c>
-      <c r="L6">
-        <v>26</v>
-      </c>
-      <c r="M6">
-        <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -3223,40 +3172,40 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="C7">
+        <v>40</v>
+      </c>
+      <c r="D7">
+        <v>51</v>
+      </c>
+      <c r="E7">
+        <v>69</v>
+      </c>
+      <c r="F7">
+        <v>65</v>
+      </c>
+      <c r="G7">
+        <v>47</v>
+      </c>
+      <c r="H7">
+        <v>50</v>
+      </c>
+      <c r="I7">
+        <v>49</v>
+      </c>
+      <c r="J7">
+        <v>51</v>
+      </c>
+      <c r="K7">
+        <v>48</v>
+      </c>
+      <c r="L7">
+        <v>44</v>
+      </c>
+      <c r="M7">
         <v>25</v>
-      </c>
-      <c r="D7">
-        <v>16</v>
-      </c>
-      <c r="E7">
-        <v>23</v>
-      </c>
-      <c r="F7">
-        <v>23</v>
-      </c>
-      <c r="G7">
-        <v>24</v>
-      </c>
-      <c r="H7">
-        <v>31</v>
-      </c>
-      <c r="I7">
-        <v>47</v>
-      </c>
-      <c r="J7">
-        <v>35</v>
-      </c>
-      <c r="K7">
-        <v>31</v>
-      </c>
-      <c r="L7">
-        <v>37</v>
-      </c>
-      <c r="M7">
-        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -3266,7 +3215,7 @@
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23.7109375" customWidth="1"/>
@@ -3329,31 +3278,40 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="B2">
+        <v>2</v>
+      </c>
       <c r="C2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D2">
         <v>2</v>
       </c>
       <c r="E2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G2">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="H2">
+        <v>6</v>
       </c>
       <c r="I2">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="J2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L2">
+        <v>3</v>
+      </c>
+      <c r="M2">
         <v>1</v>
       </c>
     </row>
@@ -3361,128 +3319,157 @@
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
+      <c r="B3">
+        <v>5</v>
+      </c>
       <c r="C3">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D3">
         <v>2</v>
       </c>
       <c r="E3">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F3">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="G3">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="H3">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I3">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="J3">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="K3">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="L3">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="M3">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="G4">
+        <v>1</v>
+      </c>
+      <c r="I4">
+        <v>2</v>
+      </c>
+      <c r="J4">
+        <v>1</v>
+      </c>
+      <c r="K4">
+        <v>1</v>
+      </c>
       <c r="L4">
+        <v>1</v>
+      </c>
+      <c r="M4">
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5">
-        <v>7</v>
-      </c>
-      <c r="C5">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D5">
-        <v>7</v>
-      </c>
-      <c r="E5">
-        <v>6</v>
-      </c>
-      <c r="F5">
-        <v>5</v>
-      </c>
-      <c r="G5">
-        <v>7</v>
-      </c>
-      <c r="H5">
-        <v>4</v>
-      </c>
-      <c r="I5">
-        <v>8</v>
-      </c>
-      <c r="J5">
-        <v>5</v>
-      </c>
-      <c r="K5">
-        <v>1</v>
-      </c>
-      <c r="L5">
-        <v>1</v>
-      </c>
-      <c r="M5">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B6">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="C6">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="D6">
         <v>11</v>
       </c>
       <c r="E6">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F6">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="G6">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="H6">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="I6">
-        <v>12</v>
+        <v>29</v>
       </c>
       <c r="J6">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="K6">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="L6">
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="M6">
-        <v>7</v>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>26</v>
+      </c>
+      <c r="C7">
+        <v>25</v>
+      </c>
+      <c r="D7">
+        <v>16</v>
+      </c>
+      <c r="E7">
+        <v>23</v>
+      </c>
+      <c r="F7">
+        <v>23</v>
+      </c>
+      <c r="G7">
+        <v>24</v>
+      </c>
+      <c r="H7">
+        <v>31</v>
+      </c>
+      <c r="I7">
+        <v>47</v>
+      </c>
+      <c r="J7">
+        <v>35</v>
+      </c>
+      <c r="K7">
+        <v>31</v>
+      </c>
+      <c r="L7">
+        <v>37</v>
+      </c>
+      <c r="M7">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -4112,7 +4099,7 @@
         <v>27</v>
       </c>
       <c r="M19">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="20" spans="1:13">
@@ -6838,7 +6825,7 @@
         <v>893</v>
       </c>
       <c r="M98">
-        <v>375</v>
+        <v>376</v>
       </c>
     </row>
   </sheetData>
@@ -6947,7 +6934,7 @@
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23.7109375" customWidth="1"/>
@@ -7014,182 +7001,156 @@
         <v>1</v>
       </c>
       <c r="D2">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G2">
-        <v>1</v>
-      </c>
-      <c r="H2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K2">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="L2">
-        <v>3</v>
-      </c>
-      <c r="M2">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B3">
-        <v>2</v>
-      </c>
       <c r="C3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D3">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="E3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F3">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G3">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="H3">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I3">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J3">
         <v>4</v>
       </c>
       <c r="K3">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="L3">
         <v>5</v>
       </c>
       <c r="M3">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B4">
-        <v>1</v>
-      </c>
-      <c r="K4">
+      <c r="L4">
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="B5">
+        <v>7</v>
+      </c>
+      <c r="C5">
+        <v>7</v>
+      </c>
+      <c r="D5">
+        <v>7</v>
+      </c>
+      <c r="E5">
+        <v>6</v>
+      </c>
+      <c r="F5">
+        <v>5</v>
       </c>
       <c r="G5">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="H5">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I5">
-        <v>1</v>
+        <v>8</v>
+      </c>
+      <c r="J5">
+        <v>5</v>
+      </c>
+      <c r="K5">
+        <v>1</v>
+      </c>
+      <c r="L5">
+        <v>1</v>
+      </c>
+      <c r="M5">
+        <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B6">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C6">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D6">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="E6">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F6">
-        <v>19</v>
+        <v>7</v>
       </c>
       <c r="G6">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="H6">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I6">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="J6">
         <v>12</v>
       </c>
       <c r="K6">
-        <v>18</v>
+        <v>3</v>
       </c>
       <c r="L6">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="M6">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
-      <c r="A7" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B7">
-        <v>8</v>
-      </c>
-      <c r="C7">
-        <v>11</v>
-      </c>
-      <c r="D7">
-        <v>29</v>
-      </c>
-      <c r="E7">
-        <v>17</v>
-      </c>
-      <c r="F7">
-        <v>26</v>
-      </c>
-      <c r="G7">
-        <v>25</v>
-      </c>
-      <c r="H7">
-        <v>13</v>
-      </c>
-      <c r="I7">
-        <v>24</v>
-      </c>
-      <c r="J7">
-        <v>21</v>
-      </c>
-      <c r="K7">
-        <v>37</v>
-      </c>
-      <c r="L7">
-        <v>27</v>
-      </c>
-      <c r="M7">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -8953,41 +8914,38 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2">
-        <v>6</v>
-      </c>
       <c r="C2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D2">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="E2">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F2">
+        <v>3</v>
+      </c>
+      <c r="G2">
+        <v>1</v>
+      </c>
+      <c r="H2">
+        <v>3</v>
+      </c>
+      <c r="I2">
+        <v>2</v>
+      </c>
+      <c r="J2">
+        <v>5</v>
+      </c>
+      <c r="K2">
         <v>8</v>
       </c>
-      <c r="G2">
-        <v>4</v>
-      </c>
-      <c r="H2">
-        <v>13</v>
-      </c>
-      <c r="I2">
-        <v>14</v>
-      </c>
-      <c r="J2">
-        <v>22</v>
-      </c>
-      <c r="K2">
-        <v>15</v>
-      </c>
       <c r="L2">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="M2">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -8995,75 +8953,51 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="C3">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="D3">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="E3">
-        <v>18</v>
+        <v>3</v>
       </c>
       <c r="F3">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="G3">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="H3">
-        <v>23</v>
+        <v>4</v>
       </c>
       <c r="I3">
-        <v>32</v>
+        <v>6</v>
       </c>
       <c r="J3">
-        <v>40</v>
+        <v>4</v>
       </c>
       <c r="K3">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="L3">
-        <v>34</v>
+        <v>5</v>
       </c>
       <c r="M3">
-        <v>16</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C4">
-        <v>2</v>
-      </c>
-      <c r="D4">
-        <v>1</v>
-      </c>
-      <c r="E4">
-        <v>2</v>
-      </c>
-      <c r="F4">
-        <v>1</v>
-      </c>
-      <c r="H4">
-        <v>2</v>
-      </c>
-      <c r="I4">
-        <v>4</v>
-      </c>
-      <c r="J4">
-        <v>3</v>
+      <c r="B4">
+        <v>1</v>
       </c>
       <c r="K4">
-        <v>2</v>
-      </c>
-      <c r="L4">
-        <v>5</v>
-      </c>
-      <c r="M4">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -9074,15 +9008,9 @@
         <v>1</v>
       </c>
       <c r="H5">
-        <v>2</v>
-      </c>
-      <c r="J5">
-        <v>2</v>
-      </c>
-      <c r="L5">
-        <v>2</v>
-      </c>
-      <c r="M5">
+        <v>1</v>
+      </c>
+      <c r="I5">
         <v>1</v>
       </c>
     </row>
@@ -9091,40 +9019,40 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="C6">
-        <v>44</v>
+        <v>9</v>
       </c>
       <c r="D6">
-        <v>49</v>
+        <v>17</v>
       </c>
       <c r="E6">
-        <v>67</v>
+        <v>13</v>
       </c>
       <c r="F6">
-        <v>69</v>
+        <v>19</v>
       </c>
       <c r="G6">
-        <v>57</v>
+        <v>15</v>
       </c>
       <c r="H6">
-        <v>80</v>
+        <v>5</v>
       </c>
       <c r="I6">
-        <v>80</v>
+        <v>15</v>
       </c>
       <c r="J6">
-        <v>64</v>
+        <v>12</v>
       </c>
       <c r="K6">
-        <v>48</v>
+        <v>18</v>
       </c>
       <c r="L6">
-        <v>44</v>
+        <v>19</v>
       </c>
       <c r="M6">
-        <v>16</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -9132,40 +9060,40 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>49</v>
+        <v>8</v>
       </c>
       <c r="C7">
-        <v>62</v>
+        <v>11</v>
       </c>
       <c r="D7">
-        <v>79</v>
+        <v>29</v>
       </c>
       <c r="E7">
-        <v>92</v>
+        <v>17</v>
       </c>
       <c r="F7">
-        <v>92</v>
+        <v>26</v>
       </c>
       <c r="G7">
-        <v>88</v>
+        <v>25</v>
       </c>
       <c r="H7">
-        <v>120</v>
+        <v>13</v>
       </c>
       <c r="I7">
-        <v>130</v>
+        <v>24</v>
       </c>
       <c r="J7">
-        <v>131</v>
+        <v>21</v>
       </c>
       <c r="K7">
-        <v>91</v>
+        <v>37</v>
       </c>
       <c r="L7">
-        <v>100</v>
+        <v>27</v>
       </c>
       <c r="M7">
-        <v>38</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -11025,10 +10953,10 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="18.7109375" customWidth="1"/>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
     <col min="2" max="2" width="4.7109375" customWidth="1"/>
     <col min="3" max="3" width="4.7109375" customWidth="1"/>
     <col min="4" max="4" width="4.7109375" customWidth="1"/>
@@ -11088,26 +11016,41 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="B2">
+        <v>6</v>
+      </c>
+      <c r="C2">
+        <v>3</v>
+      </c>
       <c r="D2">
-        <v>2</v>
+        <v>12</v>
+      </c>
+      <c r="E2">
+        <v>5</v>
+      </c>
+      <c r="F2">
+        <v>8</v>
+      </c>
+      <c r="G2">
+        <v>4</v>
       </c>
       <c r="H2">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="I2">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="J2">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="K2">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="L2">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="M2">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -11115,130 +11058,177 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="C3">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="D3">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="E3">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="F3">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="G3">
-        <v>2</v>
+        <v>26</v>
       </c>
       <c r="H3">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="I3">
-        <v>2</v>
+        <v>32</v>
       </c>
       <c r="J3">
-        <v>7</v>
+        <v>40</v>
       </c>
       <c r="K3">
-        <v>3</v>
+        <v>26</v>
       </c>
       <c r="L3">
-        <v>5</v>
+        <v>34</v>
       </c>
       <c r="M3">
-        <v>2</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C4">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4">
+        <v>2</v>
+      </c>
+      <c r="F4">
+        <v>1</v>
+      </c>
+      <c r="H4">
+        <v>2</v>
+      </c>
+      <c r="I4">
+        <v>4</v>
+      </c>
+      <c r="J4">
+        <v>3</v>
+      </c>
+      <c r="K4">
+        <v>2</v>
+      </c>
+      <c r="L4">
+        <v>5</v>
+      </c>
+      <c r="M4">
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5">
-        <v>6</v>
-      </c>
-      <c r="C5">
-        <v>4</v>
-      </c>
-      <c r="D5">
-        <v>5</v>
-      </c>
-      <c r="E5">
-        <v>4</v>
-      </c>
-      <c r="F5">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="G5">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="H5">
-        <v>4</v>
-      </c>
-      <c r="I5">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="J5">
-        <v>5</v>
-      </c>
-      <c r="K5">
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="L5">
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="M5">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B6">
-        <v>8</v>
+        <v>30</v>
       </c>
       <c r="C6">
-        <v>8</v>
+        <v>44</v>
       </c>
       <c r="D6">
-        <v>8</v>
+        <v>49</v>
       </c>
       <c r="E6">
-        <v>8</v>
+        <v>67</v>
       </c>
       <c r="F6">
-        <v>14</v>
+        <v>69</v>
       </c>
       <c r="G6">
-        <v>10</v>
+        <v>57</v>
       </c>
       <c r="H6">
-        <v>6</v>
+        <v>80</v>
       </c>
       <c r="I6">
-        <v>12</v>
+        <v>80</v>
       </c>
       <c r="J6">
-        <v>13</v>
+        <v>64</v>
       </c>
       <c r="K6">
-        <v>28</v>
+        <v>48</v>
       </c>
       <c r="L6">
-        <v>28</v>
+        <v>44</v>
       </c>
       <c r="M6">
-        <v>10</v>
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>49</v>
+      </c>
+      <c r="C7">
+        <v>62</v>
+      </c>
+      <c r="D7">
+        <v>79</v>
+      </c>
+      <c r="E7">
+        <v>92</v>
+      </c>
+      <c r="F7">
+        <v>92</v>
+      </c>
+      <c r="G7">
+        <v>88</v>
+      </c>
+      <c r="H7">
+        <v>120</v>
+      </c>
+      <c r="I7">
+        <v>130</v>
+      </c>
+      <c r="J7">
+        <v>131</v>
+      </c>
+      <c r="K7">
+        <v>91</v>
+      </c>
+      <c r="L7">
+        <v>100</v>
+      </c>
+      <c r="M7">
+        <v>38</v>
       </c>
     </row>
   </sheetData>
@@ -13154,7 +13144,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="18.7109375" customWidth="1"/>
@@ -13217,32 +13207,26 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
-      <c r="C2">
-        <v>1</v>
-      </c>
-      <c r="F2">
-        <v>1</v>
-      </c>
-      <c r="G2">
-        <v>1</v>
+      <c r="D2">
+        <v>2</v>
       </c>
       <c r="H2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J2">
         <v>1</v>
       </c>
       <c r="K2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L2">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="M2">
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -13250,19 +13234,22 @@
         <v>2</v>
       </c>
       <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3">
         <v>3</v>
       </c>
       <c r="D3">
         <v>1</v>
       </c>
       <c r="E3">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F3">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H3">
         <v>1</v>
@@ -13271,95 +13258,106 @@
         <v>2</v>
       </c>
       <c r="J3">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="K3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L3">
         <v>5</v>
       </c>
       <c r="M3">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="C4">
-        <v>8</v>
-      </c>
-      <c r="D4">
-        <v>5</v>
-      </c>
-      <c r="E4">
-        <v>5</v>
-      </c>
-      <c r="F4">
-        <v>3</v>
-      </c>
-      <c r="G4">
-        <v>2</v>
-      </c>
-      <c r="H4">
-        <v>3</v>
-      </c>
-      <c r="I4">
-        <v>2</v>
-      </c>
-      <c r="K4">
-        <v>3</v>
-      </c>
-      <c r="L4">
-        <v>6</v>
-      </c>
-      <c r="M4">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B5">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="C5">
+        <v>4</v>
+      </c>
+      <c r="D5">
+        <v>5</v>
+      </c>
+      <c r="E5">
+        <v>4</v>
+      </c>
+      <c r="F5">
+        <v>13</v>
+      </c>
+      <c r="G5">
+        <v>8</v>
+      </c>
+      <c r="H5">
+        <v>4</v>
+      </c>
+      <c r="I5">
         <v>9</v>
       </c>
-      <c r="D5">
-        <v>6</v>
-      </c>
-      <c r="E5">
-        <v>11</v>
-      </c>
-      <c r="F5">
+      <c r="J5">
+        <v>5</v>
+      </c>
+      <c r="K5">
+        <v>22</v>
+      </c>
+      <c r="L5">
+        <v>22</v>
+      </c>
+      <c r="M5">
         <v>7</v>
       </c>
-      <c r="G5">
-        <v>4</v>
-      </c>
-      <c r="H5">
-        <v>6</v>
-      </c>
-      <c r="I5">
-        <v>6</v>
-      </c>
-      <c r="J5">
-        <v>5</v>
-      </c>
-      <c r="K5">
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6">
         <v>8</v>
       </c>
-      <c r="L5">
+      <c r="C6">
+        <v>8</v>
+      </c>
+      <c r="D6">
+        <v>8</v>
+      </c>
+      <c r="E6">
+        <v>8</v>
+      </c>
+      <c r="F6">
+        <v>14</v>
+      </c>
+      <c r="G6">
+        <v>10</v>
+      </c>
+      <c r="H6">
+        <v>6</v>
+      </c>
+      <c r="I6">
+        <v>12</v>
+      </c>
+      <c r="J6">
         <v>13</v>
       </c>
-      <c r="M5">
-        <v>4</v>
+      <c r="K6">
+        <v>28</v>
+      </c>
+      <c r="L6">
+        <v>28</v>
+      </c>
+      <c r="M6">
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -15301,10 +15299,10 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:M5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="1" max="1" width="18.7109375" customWidth="1"/>
     <col min="2" max="2" width="4.7109375" customWidth="1"/>
     <col min="3" max="3" width="4.7109375" customWidth="1"/>
     <col min="4" max="4" width="4.7109375" customWidth="1"/>
@@ -15364,32 +15362,32 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
       <c r="C2">
         <v>1</v>
       </c>
-      <c r="D2">
-        <v>2</v>
-      </c>
-      <c r="E2">
-        <v>1</v>
-      </c>
       <c r="F2">
-        <v>3</v>
+        <v>1</v>
+      </c>
+      <c r="G2">
+        <v>1</v>
+      </c>
+      <c r="H2">
+        <v>2</v>
       </c>
       <c r="I2">
         <v>2</v>
       </c>
       <c r="J2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L2">
-        <v>3</v>
-      </c>
-      <c r="M2">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -15397,10 +15395,7 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>1</v>
-      </c>
-      <c r="C3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D3">
         <v>1</v>
@@ -15409,118 +15404,107 @@
         <v>6</v>
       </c>
       <c r="F3">
+        <v>3</v>
+      </c>
+      <c r="G3">
         <v>1</v>
       </c>
       <c r="H3">
         <v>1</v>
       </c>
       <c r="I3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J3">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K3">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L3">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M3">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4">
+        <v>13</v>
+      </c>
+      <c r="C4">
+        <v>8</v>
+      </c>
+      <c r="D4">
+        <v>5</v>
+      </c>
+      <c r="E4">
+        <v>5</v>
+      </c>
+      <c r="F4">
+        <v>3</v>
+      </c>
+      <c r="G4">
+        <v>2</v>
+      </c>
+      <c r="H4">
         <v>3</v>
       </c>
       <c r="I4">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="K4">
+        <v>3</v>
+      </c>
+      <c r="L4">
+        <v>6</v>
       </c>
       <c r="M4">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B5">
-        <v>5</v>
+        <v>17</v>
       </c>
       <c r="C5">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D5">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E5">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="F5">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="G5">
         <v>4</v>
       </c>
       <c r="H5">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I5">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="J5">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="K5">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="L5">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="M5">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
-      <c r="A6" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6">
-        <v>6</v>
-      </c>
-      <c r="C6">
-        <v>8</v>
-      </c>
-      <c r="D6">
-        <v>7</v>
-      </c>
-      <c r="E6">
-        <v>12</v>
-      </c>
-      <c r="F6">
-        <v>19</v>
-      </c>
-      <c r="G6">
-        <v>4</v>
-      </c>
-      <c r="H6">
-        <v>8</v>
-      </c>
-      <c r="I6">
-        <v>15</v>
-      </c>
-      <c r="J6">
-        <v>21</v>
-      </c>
-      <c r="K6">
-        <v>16</v>
-      </c>
-      <c r="L6">
-        <v>28</v>
-      </c>
-      <c r="M6">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -17275,7 +17259,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23.7109375" customWidth="1"/>
@@ -17338,41 +17322,32 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2">
-        <v>4</v>
-      </c>
       <c r="C2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E2">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F2">
-        <v>9</v>
-      </c>
-      <c r="G2">
-        <v>3</v>
-      </c>
-      <c r="H2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J2">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="K2">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="L2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M2">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -17380,60 +17355,45 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C3">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D3">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E3">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F3">
-        <v>6</v>
-      </c>
-      <c r="G3">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="H3">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="I3">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="J3">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="K3">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="L3">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="M3">
-        <v>9</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B4">
-        <v>1</v>
-      </c>
-      <c r="D4">
-        <v>1</v>
-      </c>
-      <c r="E4">
-        <v>1</v>
-      </c>
-      <c r="J4">
-        <v>3</v>
-      </c>
-      <c r="K4">
-        <v>2</v>
+      <c r="I4">
+        <v>1</v>
       </c>
       <c r="M4">
         <v>1</v>
@@ -17441,92 +17401,84 @@
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="B5">
+        <v>5</v>
+      </c>
+      <c r="C5">
+        <v>6</v>
+      </c>
+      <c r="D5">
+        <v>4</v>
+      </c>
+      <c r="E5">
+        <v>5</v>
+      </c>
+      <c r="F5">
+        <v>15</v>
+      </c>
+      <c r="G5">
+        <v>4</v>
+      </c>
+      <c r="H5">
+        <v>7</v>
+      </c>
+      <c r="I5">
+        <v>11</v>
+      </c>
+      <c r="J5">
+        <v>15</v>
       </c>
       <c r="K5">
-        <v>1</v>
+        <v>11</v>
+      </c>
+      <c r="L5">
+        <v>19</v>
+      </c>
+      <c r="M5">
+        <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B6">
-        <v>23</v>
+        <v>6</v>
       </c>
       <c r="C6">
-        <v>31</v>
+        <v>8</v>
       </c>
       <c r="D6">
-        <v>22</v>
+        <v>7</v>
       </c>
       <c r="E6">
-        <v>44</v>
+        <v>12</v>
       </c>
       <c r="F6">
-        <v>38</v>
+        <v>19</v>
       </c>
       <c r="G6">
-        <v>24</v>
+        <v>4</v>
       </c>
       <c r="H6">
-        <v>50</v>
+        <v>8</v>
       </c>
       <c r="I6">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="J6">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="K6">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="L6">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="M6">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
-      <c r="A7" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B7">
-        <v>32</v>
-      </c>
-      <c r="C7">
-        <v>40</v>
-      </c>
-      <c r="D7">
-        <v>32</v>
-      </c>
-      <c r="E7">
-        <v>57</v>
-      </c>
-      <c r="F7">
-        <v>53</v>
-      </c>
-      <c r="G7">
-        <v>34</v>
-      </c>
-      <c r="H7">
-        <v>63</v>
-      </c>
-      <c r="I7">
-        <v>44</v>
-      </c>
-      <c r="J7">
-        <v>47</v>
-      </c>
-      <c r="K7">
-        <v>46</v>
-      </c>
-      <c r="L7">
-        <v>33</v>
-      </c>
-      <c r="M7">
-        <v>31</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -19052,7 +19004,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23.7109375" customWidth="1"/>
@@ -19115,32 +19067,41 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="B2">
+        <v>4</v>
+      </c>
       <c r="C2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D2">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="E2">
+        <v>5</v>
       </c>
       <c r="F2">
-        <v>2</v>
+        <v>9</v>
+      </c>
+      <c r="G2">
+        <v>3</v>
       </c>
       <c r="H2">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I2">
         <v>4</v>
       </c>
       <c r="J2">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="K2">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L2">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M2">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -19150,35 +19111,38 @@
       <c r="B3">
         <v>4</v>
       </c>
+      <c r="C3">
+        <v>5</v>
+      </c>
       <c r="D3">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E3">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="F3">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="G3">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="H3">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="I3">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J3">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="K3">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="L3">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="M3">
-        <v>1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -19188,14 +19152,17 @@
       <c r="B4">
         <v>1</v>
       </c>
-      <c r="H4">
-        <v>2</v>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4">
+        <v>1</v>
+      </c>
+      <c r="J4">
+        <v>3</v>
       </c>
       <c r="K4">
-        <v>3</v>
-      </c>
-      <c r="L4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M4">
         <v>1</v>
@@ -19203,84 +19170,92 @@
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5">
-        <v>5</v>
-      </c>
-      <c r="C5">
-        <v>7</v>
-      </c>
-      <c r="D5">
-        <v>11</v>
-      </c>
-      <c r="E5">
-        <v>21</v>
-      </c>
-      <c r="F5">
-        <v>25</v>
-      </c>
-      <c r="G5">
-        <v>15</v>
-      </c>
-      <c r="H5">
-        <v>10</v>
-      </c>
-      <c r="I5">
-        <v>9</v>
-      </c>
-      <c r="J5">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="K5">
-        <v>18</v>
-      </c>
-      <c r="L5">
-        <v>11</v>
-      </c>
-      <c r="M5">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B6">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="C6">
-        <v>10</v>
+        <v>31</v>
       </c>
       <c r="D6">
+        <v>22</v>
+      </c>
+      <c r="E6">
+        <v>44</v>
+      </c>
+      <c r="F6">
+        <v>38</v>
+      </c>
+      <c r="G6">
+        <v>24</v>
+      </c>
+      <c r="H6">
+        <v>50</v>
+      </c>
+      <c r="I6">
+        <v>34</v>
+      </c>
+      <c r="J6">
+        <v>26</v>
+      </c>
+      <c r="K6">
+        <v>24</v>
+      </c>
+      <c r="L6">
         <v>14</v>
       </c>
-      <c r="E6">
-        <v>23</v>
-      </c>
-      <c r="F6">
-        <v>28</v>
-      </c>
-      <c r="G6">
-        <v>16</v>
-      </c>
-      <c r="H6">
-        <v>14</v>
-      </c>
-      <c r="I6">
-        <v>17</v>
-      </c>
-      <c r="J6">
-        <v>16</v>
-      </c>
-      <c r="K6">
+      <c r="M6">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>32</v>
+      </c>
+      <c r="C7">
+        <v>40</v>
+      </c>
+      <c r="D7">
+        <v>32</v>
+      </c>
+      <c r="E7">
+        <v>57</v>
+      </c>
+      <c r="F7">
+        <v>53</v>
+      </c>
+      <c r="G7">
+        <v>34</v>
+      </c>
+      <c r="H7">
+        <v>63</v>
+      </c>
+      <c r="I7">
+        <v>44</v>
+      </c>
+      <c r="J7">
+        <v>47</v>
+      </c>
+      <c r="K7">
+        <v>46</v>
+      </c>
+      <c r="L7">
+        <v>33</v>
+      </c>
+      <c r="M7">
         <v>31</v>
-      </c>
-      <c r="L6">
-        <v>22</v>
-      </c>
-      <c r="M6">
-        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -20306,7 +20281,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23.7109375" customWidth="1"/>
@@ -20370,22 +20345,31 @@
         <v>1</v>
       </c>
       <c r="C2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D2">
         <v>1</v>
       </c>
+      <c r="F2">
+        <v>2</v>
+      </c>
       <c r="H2">
         <v>1</v>
       </c>
       <c r="I2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J2">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="K2">
+        <v>5</v>
       </c>
       <c r="L2">
-        <v>1</v>
+        <v>4</v>
+      </c>
+      <c r="M2">
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -20393,123 +20377,139 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D3">
         <v>2</v>
       </c>
+      <c r="E3">
+        <v>2</v>
+      </c>
       <c r="F3">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G3">
         <v>1</v>
       </c>
       <c r="H3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I3">
-        <v>2</v>
+        <v>4</v>
+      </c>
+      <c r="J3">
+        <v>4</v>
       </c>
       <c r="K3">
-        <v>2</v>
+        <v>5</v>
+      </c>
+      <c r="L3">
+        <v>6</v>
       </c>
       <c r="M3">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="J4">
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="H4">
+        <v>2</v>
+      </c>
+      <c r="K4">
+        <v>3</v>
+      </c>
+      <c r="L4">
+        <v>1</v>
+      </c>
+      <c r="M4">
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="B5">
+        <v>5</v>
+      </c>
+      <c r="C5">
+        <v>7</v>
+      </c>
+      <c r="D5">
+        <v>11</v>
+      </c>
+      <c r="E5">
+        <v>21</v>
+      </c>
+      <c r="F5">
+        <v>25</v>
+      </c>
+      <c r="G5">
+        <v>15</v>
+      </c>
+      <c r="H5">
+        <v>10</v>
+      </c>
+      <c r="I5">
+        <v>9</v>
+      </c>
+      <c r="J5">
+        <v>11</v>
       </c>
       <c r="K5">
-        <v>1</v>
+        <v>18</v>
+      </c>
+      <c r="L5">
+        <v>11</v>
+      </c>
+      <c r="M5">
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B6">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C6">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D6">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="E6">
-        <v>5</v>
+        <v>23</v>
       </c>
       <c r="F6">
-        <v>5</v>
+        <v>28</v>
       </c>
       <c r="G6">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="H6">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="I6">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="J6">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="K6">
-        <v>4</v>
+        <v>31</v>
       </c>
       <c r="L6">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
-      <c r="A7" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B7">
-        <v>8</v>
-      </c>
-      <c r="C7">
-        <v>7</v>
-      </c>
-      <c r="D7">
-        <v>8</v>
-      </c>
-      <c r="E7">
-        <v>5</v>
-      </c>
-      <c r="F7">
-        <v>8</v>
-      </c>
-      <c r="G7">
-        <v>2</v>
-      </c>
-      <c r="H7">
-        <v>8</v>
-      </c>
-      <c r="I7">
-        <v>7</v>
-      </c>
-      <c r="J7">
-        <v>4</v>
-      </c>
-      <c r="K7">
-        <v>7</v>
-      </c>
-      <c r="L7">
-        <v>7</v>
-      </c>
-      <c r="M7">
-        <v>2</v>
+        <v>22</v>
+      </c>
+      <c r="M6">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add data for 2026-09-01
</commit_message>
<xml_diff>
--- a/output/cta-violent-crime-full-year.xlsx
+++ b/output/cta-violent-crime-full-year.xlsx
@@ -9,17 +9,17 @@
   <sheets>
     <sheet name="Citywide Totals" sheetId="1" r:id="rId1"/>
     <sheet name="By Neighborhood" sheetId="2" r:id="rId2"/>
-    <sheet name="Greektown" sheetId="3" r:id="rId3"/>
-    <sheet name="Edgewater" sheetId="4" r:id="rId4"/>
-    <sheet name="Little Italy, UIC" sheetId="5" r:id="rId5"/>
-    <sheet name="Austin" sheetId="6" r:id="rId6"/>
-    <sheet name="Washington Heights" sheetId="7" r:id="rId7"/>
-    <sheet name="Gage Park" sheetId="8" r:id="rId8"/>
-    <sheet name="Humboldt Park" sheetId="9" r:id="rId9"/>
-    <sheet name="Grand Crossing" sheetId="10" r:id="rId10"/>
-    <sheet name="Lower West Side" sheetId="11" r:id="rId11"/>
-    <sheet name="Near South Side" sheetId="12" r:id="rId12"/>
-    <sheet name="Englewood" sheetId="13" r:id="rId13"/>
+    <sheet name="Englewood" sheetId="3" r:id="rId3"/>
+    <sheet name="Greektown" sheetId="4" r:id="rId4"/>
+    <sheet name="Edgewater" sheetId="5" r:id="rId5"/>
+    <sheet name="Little Italy, UIC" sheetId="6" r:id="rId6"/>
+    <sheet name="Austin" sheetId="7" r:id="rId7"/>
+    <sheet name="Washington Heights" sheetId="8" r:id="rId8"/>
+    <sheet name="Gage Park" sheetId="9" r:id="rId9"/>
+    <sheet name="Humboldt Park" sheetId="10" r:id="rId10"/>
+    <sheet name="Grand Crossing" sheetId="11" r:id="rId11"/>
+    <sheet name="Lower West Side" sheetId="12" r:id="rId12"/>
+    <sheet name="Near South Side" sheetId="13" r:id="rId13"/>
     <sheet name="Loop" sheetId="14" r:id="rId14"/>
     <sheet name="Sheffield &amp; DePaul" sheetId="15" r:id="rId15"/>
     <sheet name="Roseland" sheetId="16" r:id="rId16"/>
@@ -880,7 +880,7 @@
         <v>121</v>
       </c>
       <c r="J2">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K2">
         <v>154</v>
@@ -889,7 +889,7 @@
         <v>137</v>
       </c>
       <c r="M2">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -915,16 +915,16 @@
         <v>150</v>
       </c>
       <c r="H3">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="I3">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="J3">
         <v>244</v>
       </c>
       <c r="K3">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="L3">
         <v>262</v>
@@ -950,28 +950,28 @@
         <v>11</v>
       </c>
       <c r="F4">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H4">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="I4">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="J4">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="K4">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="L4">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="M4">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -1070,28 +1070,28 @@
         <v>761</v>
       </c>
       <c r="F7">
-        <v>848</v>
+        <v>849</v>
       </c>
       <c r="G7">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="H7">
-        <v>776</v>
+        <v>779</v>
       </c>
       <c r="I7">
-        <v>874</v>
+        <v>876</v>
       </c>
       <c r="J7">
-        <v>838</v>
+        <v>840</v>
       </c>
       <c r="K7">
-        <v>958</v>
+        <v>961</v>
       </c>
       <c r="L7">
-        <v>893</v>
+        <v>896</v>
       </c>
       <c r="M7">
-        <v>421</v>
+        <v>424</v>
       </c>
     </row>
   </sheetData>
@@ -1100,6 +1100,241 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:M6"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="18.7109375" customWidth="1"/>
+    <col min="2" max="2" width="4.7109375" customWidth="1"/>
+    <col min="3" max="3" width="4.7109375" customWidth="1"/>
+    <col min="4" max="4" width="4.7109375" customWidth="1"/>
+    <col min="5" max="5" width="4.7109375" customWidth="1"/>
+    <col min="6" max="6" width="4.7109375" customWidth="1"/>
+    <col min="7" max="7" width="4.7109375" customWidth="1"/>
+    <col min="8" max="8" width="4.7109375" customWidth="1"/>
+    <col min="9" max="9" width="4.7109375" customWidth="1"/>
+    <col min="10" max="10" width="4.7109375" customWidth="1"/>
+    <col min="11" max="11" width="4.7109375" customWidth="1"/>
+    <col min="12" max="12" width="4.7109375" customWidth="1"/>
+    <col min="13" max="13" width="4.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1">
+        <v>2015</v>
+      </c>
+      <c r="C1" s="1">
+        <v>2016</v>
+      </c>
+      <c r="D1" s="1">
+        <v>2017</v>
+      </c>
+      <c r="E1" s="1">
+        <v>2018</v>
+      </c>
+      <c r="F1" s="1">
+        <v>2019</v>
+      </c>
+      <c r="G1" s="1">
+        <v>2020</v>
+      </c>
+      <c r="H1" s="1">
+        <v>2021</v>
+      </c>
+      <c r="I1" s="1">
+        <v>2022</v>
+      </c>
+      <c r="J1" s="1">
+        <v>2023</v>
+      </c>
+      <c r="K1" s="1">
+        <v>2024</v>
+      </c>
+      <c r="L1" s="1">
+        <v>2025</v>
+      </c>
+      <c r="M1" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+      <c r="G2">
+        <v>4</v>
+      </c>
+      <c r="H2">
+        <v>1</v>
+      </c>
+      <c r="I2">
+        <v>1</v>
+      </c>
+      <c r="J2">
+        <v>1</v>
+      </c>
+      <c r="K2">
+        <v>4</v>
+      </c>
+      <c r="L2">
+        <v>2</v>
+      </c>
+      <c r="M2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <v>2</v>
+      </c>
+      <c r="F3">
+        <v>2</v>
+      </c>
+      <c r="G3">
+        <v>2</v>
+      </c>
+      <c r="H3">
+        <v>4</v>
+      </c>
+      <c r="I3">
+        <v>5</v>
+      </c>
+      <c r="J3">
+        <v>7</v>
+      </c>
+      <c r="K3">
+        <v>2</v>
+      </c>
+      <c r="L3">
+        <v>2</v>
+      </c>
+      <c r="M3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="K4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5">
+        <v>6</v>
+      </c>
+      <c r="C5">
+        <v>8</v>
+      </c>
+      <c r="D5">
+        <v>6</v>
+      </c>
+      <c r="E5">
+        <v>7</v>
+      </c>
+      <c r="F5">
+        <v>3</v>
+      </c>
+      <c r="G5">
+        <v>5</v>
+      </c>
+      <c r="H5">
+        <v>1</v>
+      </c>
+      <c r="I5">
+        <v>7</v>
+      </c>
+      <c r="J5">
+        <v>11</v>
+      </c>
+      <c r="K5">
+        <v>8</v>
+      </c>
+      <c r="L5">
+        <v>5</v>
+      </c>
+      <c r="M5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6">
+        <v>8</v>
+      </c>
+      <c r="C6">
+        <v>10</v>
+      </c>
+      <c r="D6">
+        <v>8</v>
+      </c>
+      <c r="E6">
+        <v>10</v>
+      </c>
+      <c r="F6">
+        <v>6</v>
+      </c>
+      <c r="G6">
+        <v>11</v>
+      </c>
+      <c r="H6">
+        <v>6</v>
+      </c>
+      <c r="I6">
+        <v>13</v>
+      </c>
+      <c r="J6">
+        <v>19</v>
+      </c>
+      <c r="K6">
+        <v>15</v>
+      </c>
+      <c r="L6">
+        <v>9</v>
+      </c>
+      <c r="M6">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1363,7 +1598,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M5"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1556,231 +1791,6 @@
       </c>
       <c r="M5">
         <v>5</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M7"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
-    <col min="2" max="2" width="4.7109375" customWidth="1"/>
-    <col min="3" max="3" width="4.7109375" customWidth="1"/>
-    <col min="4" max="4" width="4.7109375" customWidth="1"/>
-    <col min="5" max="5" width="4.7109375" customWidth="1"/>
-    <col min="6" max="6" width="4.7109375" customWidth="1"/>
-    <col min="7" max="7" width="4.7109375" customWidth="1"/>
-    <col min="8" max="8" width="4.7109375" customWidth="1"/>
-    <col min="9" max="9" width="4.7109375" customWidth="1"/>
-    <col min="10" max="10" width="4.7109375" customWidth="1"/>
-    <col min="11" max="11" width="4.7109375" customWidth="1"/>
-    <col min="12" max="12" width="4.7109375" customWidth="1"/>
-    <col min="13" max="13" width="4.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:13">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1">
-        <v>2015</v>
-      </c>
-      <c r="C1" s="1">
-        <v>2016</v>
-      </c>
-      <c r="D1" s="1">
-        <v>2017</v>
-      </c>
-      <c r="E1" s="1">
-        <v>2018</v>
-      </c>
-      <c r="F1" s="1">
-        <v>2019</v>
-      </c>
-      <c r="G1" s="1">
-        <v>2020</v>
-      </c>
-      <c r="H1" s="1">
-        <v>2021</v>
-      </c>
-      <c r="I1" s="1">
-        <v>2022</v>
-      </c>
-      <c r="J1" s="1">
-        <v>2023</v>
-      </c>
-      <c r="K1" s="1">
-        <v>2024</v>
-      </c>
-      <c r="L1" s="1">
-        <v>2025</v>
-      </c>
-      <c r="M1" s="1">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="F2">
-        <v>1</v>
-      </c>
-      <c r="G2">
-        <v>2</v>
-      </c>
-      <c r="H2">
-        <v>1</v>
-      </c>
-      <c r="I2">
-        <v>2</v>
-      </c>
-      <c r="J2">
-        <v>2</v>
-      </c>
-      <c r="K2">
-        <v>3</v>
-      </c>
-      <c r="M2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
-      <c r="A3" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3">
-        <v>1</v>
-      </c>
-      <c r="C3">
-        <v>1</v>
-      </c>
-      <c r="D3">
-        <v>1</v>
-      </c>
-      <c r="E3">
-        <v>2</v>
-      </c>
-      <c r="G3">
-        <v>2</v>
-      </c>
-      <c r="H3">
-        <v>2</v>
-      </c>
-      <c r="I3">
-        <v>3</v>
-      </c>
-      <c r="J3">
-        <v>1</v>
-      </c>
-      <c r="K3">
-        <v>1</v>
-      </c>
-      <c r="M3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
-      <c r="A4" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="J4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
-      <c r="A5" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="K5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
-      <c r="A6" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B6">
-        <v>6</v>
-      </c>
-      <c r="C6">
-        <v>2</v>
-      </c>
-      <c r="D6">
-        <v>5</v>
-      </c>
-      <c r="E6">
-        <v>5</v>
-      </c>
-      <c r="F6">
-        <v>4</v>
-      </c>
-      <c r="G6">
-        <v>4</v>
-      </c>
-      <c r="H6">
-        <v>6</v>
-      </c>
-      <c r="I6">
-        <v>8</v>
-      </c>
-      <c r="J6">
-        <v>4</v>
-      </c>
-      <c r="K6">
-        <v>3</v>
-      </c>
-      <c r="L6">
-        <v>4</v>
-      </c>
-      <c r="M6">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
-      <c r="A7" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B7">
-        <v>7</v>
-      </c>
-      <c r="C7">
-        <v>3</v>
-      </c>
-      <c r="D7">
-        <v>6</v>
-      </c>
-      <c r="E7">
-        <v>7</v>
-      </c>
-      <c r="F7">
-        <v>5</v>
-      </c>
-      <c r="G7">
-        <v>8</v>
-      </c>
-      <c r="H7">
-        <v>9</v>
-      </c>
-      <c r="I7">
-        <v>13</v>
-      </c>
-      <c r="J7">
-        <v>8</v>
-      </c>
-      <c r="K7">
-        <v>8</v>
-      </c>
-      <c r="L7">
-        <v>4</v>
-      </c>
-      <c r="M7">
-        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -1853,38 +1863,26 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C2">
-        <v>1</v>
-      </c>
-      <c r="D2">
-        <v>6</v>
-      </c>
-      <c r="E2">
-        <v>1</v>
-      </c>
       <c r="F2">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="G2">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="H2">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="I2">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="J2">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="K2">
         <v>3</v>
       </c>
-      <c r="L2">
-        <v>6</v>
-      </c>
       <c r="M2">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -1892,76 +1890,49 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C3">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D3">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="E3">
-        <v>10</v>
-      </c>
-      <c r="F3">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="G3">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="H3">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="I3">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="J3">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="K3">
-        <v>20</v>
-      </c>
-      <c r="L3">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="M3">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B4">
-        <v>1</v>
-      </c>
-      <c r="D4">
-        <v>1</v>
-      </c>
-      <c r="H4">
-        <v>2</v>
-      </c>
       <c r="J4">
         <v>1</v>
-      </c>
-      <c r="K4">
-        <v>1</v>
-      </c>
-      <c r="L4">
-        <v>1</v>
-      </c>
-      <c r="M4">
-        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="H5">
-        <v>1</v>
-      </c>
-      <c r="I5">
+      <c r="K5">
         <v>1</v>
       </c>
     </row>
@@ -1970,40 +1941,40 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>34</v>
+        <v>6</v>
       </c>
       <c r="C6">
-        <v>45</v>
+        <v>2</v>
       </c>
       <c r="D6">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="E6">
-        <v>22</v>
+        <v>5</v>
       </c>
       <c r="F6">
-        <v>42</v>
+        <v>4</v>
       </c>
       <c r="G6">
-        <v>32</v>
+        <v>4</v>
       </c>
       <c r="H6">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="I6">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="J6">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="K6">
-        <v>44</v>
+        <v>3</v>
       </c>
       <c r="L6">
-        <v>44</v>
+        <v>4</v>
       </c>
       <c r="M6">
-        <v>15</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -2011,40 +1982,40 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>40</v>
+        <v>7</v>
       </c>
       <c r="C7">
-        <v>51</v>
+        <v>3</v>
       </c>
       <c r="D7">
-        <v>50</v>
+        <v>6</v>
       </c>
       <c r="E7">
-        <v>33</v>
+        <v>7</v>
       </c>
       <c r="F7">
-        <v>63</v>
+        <v>5</v>
       </c>
       <c r="G7">
-        <v>50</v>
+        <v>8</v>
       </c>
       <c r="H7">
-        <v>47</v>
+        <v>9</v>
       </c>
       <c r="I7">
-        <v>45</v>
+        <v>13</v>
       </c>
       <c r="J7">
-        <v>37</v>
+        <v>8</v>
       </c>
       <c r="K7">
-        <v>68</v>
+        <v>8</v>
       </c>
       <c r="L7">
-        <v>71</v>
+        <v>4</v>
       </c>
       <c r="M7">
-        <v>25</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -4444,7 +4415,7 @@
         <v>71</v>
       </c>
       <c r="M28">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="29" spans="1:13">
@@ -5518,25 +5489,28 @@
         <v>4</v>
       </c>
       <c r="F61">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G61">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H61">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="I61">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J61">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K61">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="L61">
-        <v>3</v>
+        <v>6</v>
+      </c>
+      <c r="M61">
+        <v>2</v>
       </c>
     </row>
     <row r="62" spans="1:13">
@@ -6846,28 +6820,28 @@
         <v>761</v>
       </c>
       <c r="F98">
-        <v>848</v>
+        <v>849</v>
       </c>
       <c r="G98">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="H98">
-        <v>776</v>
+        <v>779</v>
       </c>
       <c r="I98">
-        <v>874</v>
+        <v>876</v>
       </c>
       <c r="J98">
-        <v>838</v>
+        <v>840</v>
       </c>
       <c r="K98">
-        <v>958</v>
+        <v>961</v>
       </c>
       <c r="L98">
-        <v>893</v>
+        <v>896</v>
       </c>
       <c r="M98">
-        <v>421</v>
+        <v>424</v>
       </c>
     </row>
   </sheetData>
@@ -9048,7 +9022,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23.7109375" customWidth="1"/>
@@ -9063,159 +9037,246 @@
     <col min="10" max="10" width="4.7109375" customWidth="1"/>
     <col min="11" max="11" width="4.7109375" customWidth="1"/>
     <col min="12" max="12" width="4.7109375" customWidth="1"/>
+    <col min="13" max="13" width="4.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12">
+    <row r="1" spans="1:13">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1">
+        <v>2015</v>
+      </c>
+      <c r="C1" s="1">
         <v>2016</v>
       </c>
-      <c r="C1" s="1">
+      <c r="D1" s="1">
         <v>2017</v>
       </c>
-      <c r="D1" s="1">
+      <c r="E1" s="1">
         <v>2018</v>
       </c>
-      <c r="E1" s="1">
+      <c r="F1" s="1">
         <v>2019</v>
       </c>
-      <c r="F1" s="1">
+      <c r="G1" s="1">
         <v>2020</v>
       </c>
-      <c r="G1" s="1">
+      <c r="H1" s="1">
         <v>2021</v>
       </c>
-      <c r="H1" s="1">
+      <c r="I1" s="1">
         <v>2022</v>
       </c>
-      <c r="I1" s="1">
+      <c r="J1" s="1">
         <v>2023</v>
       </c>
-      <c r="J1" s="1">
+      <c r="K1" s="1">
         <v>2024</v>
       </c>
-      <c r="K1" s="1">
+      <c r="L1" s="1">
         <v>2025</v>
       </c>
-      <c r="L1" s="1">
+      <c r="M1" s="1">
         <v>2026</v>
       </c>
     </row>
-    <row r="2" spans="1:12">
+    <row r="2" spans="1:13">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
       <c r="C2">
         <v>1</v>
       </c>
+      <c r="D2">
+        <v>6</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2">
+        <v>9</v>
+      </c>
+      <c r="G2">
+        <v>7</v>
+      </c>
+      <c r="H2">
+        <v>11</v>
+      </c>
+      <c r="I2">
+        <v>10</v>
+      </c>
       <c r="J2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12">
+        <v>9</v>
+      </c>
+      <c r="K2">
+        <v>3</v>
+      </c>
+      <c r="L2">
+        <v>6</v>
+      </c>
+      <c r="M2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B3">
-        <v>1</v>
+        <v>5</v>
+      </c>
+      <c r="C3">
+        <v>5</v>
+      </c>
+      <c r="D3">
+        <v>18</v>
+      </c>
+      <c r="E3">
+        <v>10</v>
       </c>
       <c r="F3">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="G3">
-        <v>1</v>
+        <v>11</v>
+      </c>
+      <c r="H3">
+        <v>7</v>
+      </c>
+      <c r="I3">
+        <v>13</v>
+      </c>
+      <c r="J3">
+        <v>12</v>
       </c>
       <c r="K3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12">
+        <v>20</v>
+      </c>
+      <c r="L3">
+        <v>20</v>
+      </c>
+      <c r="M3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
       <c r="D4">
         <v>1</v>
       </c>
+      <c r="H4">
+        <v>2</v>
+      </c>
       <c r="J4">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:12">
+      <c r="K4">
+        <v>1</v>
+      </c>
+      <c r="L4">
+        <v>1</v>
+      </c>
+      <c r="M4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C5">
-        <v>1</v>
-      </c>
-      <c r="D5">
-        <v>4</v>
-      </c>
-      <c r="E5">
-        <v>5</v>
-      </c>
-      <c r="F5">
-        <v>3</v>
-      </c>
-      <c r="G5">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H5">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I5">
         <v>1</v>
       </c>
-      <c r="J5">
-        <v>2</v>
-      </c>
-      <c r="K5">
-        <v>1</v>
-      </c>
-      <c r="L5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12">
+    </row>
+    <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B6">
-        <v>2</v>
+        <v>34</v>
       </c>
       <c r="C6">
-        <v>2</v>
+        <v>45</v>
       </c>
       <c r="D6">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="E6">
-        <v>5</v>
+        <v>22</v>
       </c>
       <c r="F6">
-        <v>4</v>
+        <v>42</v>
       </c>
       <c r="G6">
-        <v>2</v>
+        <v>32</v>
       </c>
       <c r="H6">
-        <v>5</v>
+        <v>26</v>
       </c>
       <c r="I6">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="J6">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="K6">
-        <v>2</v>
+        <v>44</v>
       </c>
       <c r="L6">
-        <v>2</v>
+        <v>44</v>
+      </c>
+      <c r="M6">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>40</v>
+      </c>
+      <c r="C7">
+        <v>51</v>
+      </c>
+      <c r="D7">
+        <v>50</v>
+      </c>
+      <c r="E7">
+        <v>33</v>
+      </c>
+      <c r="F7">
+        <v>63</v>
+      </c>
+      <c r="G7">
+        <v>50</v>
+      </c>
+      <c r="H7">
+        <v>47</v>
+      </c>
+      <c r="I7">
+        <v>45</v>
+      </c>
+      <c r="J7">
+        <v>37</v>
+      </c>
+      <c r="K7">
+        <v>68</v>
+      </c>
+      <c r="L7">
+        <v>71</v>
+      </c>
+      <c r="M7">
+        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -11319,7 +11380,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23.7109375" customWidth="1"/>
@@ -11334,202 +11395,159 @@
     <col min="10" max="10" width="4.7109375" customWidth="1"/>
     <col min="11" max="11" width="4.7109375" customWidth="1"/>
     <col min="12" max="12" width="4.7109375" customWidth="1"/>
-    <col min="13" max="13" width="4.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1">
-        <v>2015</v>
+        <v>2016</v>
       </c>
       <c r="C1" s="1">
-        <v>2016</v>
+        <v>2017</v>
       </c>
       <c r="D1" s="1">
-        <v>2017</v>
+        <v>2018</v>
       </c>
       <c r="E1" s="1">
-        <v>2018</v>
+        <v>2019</v>
       </c>
       <c r="F1" s="1">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="G1" s="1">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="H1" s="1">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="I1" s="1">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="J1" s="1">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="K1" s="1">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L1" s="1">
-        <v>2025</v>
-      </c>
-      <c r="M1" s="1">
         <v>2026</v>
       </c>
     </row>
-    <row r="2" spans="1:13">
+    <row r="2" spans="1:12">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
       <c r="C2">
         <v>1</v>
       </c>
-      <c r="D2">
-        <v>2</v>
-      </c>
-      <c r="F2">
-        <v>3</v>
-      </c>
-      <c r="G2">
-        <v>3</v>
-      </c>
-      <c r="I2">
-        <v>2</v>
-      </c>
       <c r="J2">
         <v>1</v>
       </c>
-      <c r="K2">
-        <v>5</v>
-      </c>
-      <c r="L2">
-        <v>3</v>
-      </c>
-      <c r="M2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
+    </row>
+    <row r="3" spans="1:12">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D3">
-        <v>1</v>
-      </c>
-      <c r="E3">
+      <c r="B3">
         <v>1</v>
       </c>
       <c r="F3">
         <v>1</v>
       </c>
       <c r="G3">
-        <v>4</v>
-      </c>
-      <c r="H3">
-        <v>1</v>
-      </c>
-      <c r="I3">
-        <v>3</v>
-      </c>
-      <c r="J3">
-        <v>3</v>
-      </c>
-      <c r="L3">
-        <v>2</v>
-      </c>
-      <c r="M3">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
+        <v>1</v>
+      </c>
+      <c r="K3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="M4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="J4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12">
       <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B5">
-        <v>4</v>
-      </c>
       <c r="C5">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D5">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E5">
         <v>5</v>
       </c>
       <c r="F5">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G5">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H5">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="I5">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="J5">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="K5">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="L5">
-        <v>8</v>
-      </c>
-      <c r="M5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12">
       <c r="A6" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B6">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C6">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D6">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="E6">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F6">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="G6">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="H6">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="I6">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="J6">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="K6">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="L6">
-        <v>13</v>
-      </c>
-      <c r="M6">
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -13320,19 +13338,19 @@
         <v>1</v>
       </c>
       <c r="C2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F2">
-        <v>2</v>
-      </c>
-      <c r="H2">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="G2">
+        <v>3</v>
       </c>
       <c r="I2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -13341,66 +13359,48 @@
         <v>5</v>
       </c>
       <c r="L2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M2">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B3">
-        <v>4</v>
-      </c>
       <c r="D3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F3">
         <v>1</v>
       </c>
       <c r="G3">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H3">
         <v>1</v>
       </c>
       <c r="I3">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J3">
-        <v>4</v>
-      </c>
-      <c r="K3">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L3">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="M3">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B4">
-        <v>1</v>
-      </c>
-      <c r="H4">
-        <v>2</v>
-      </c>
-      <c r="K4">
-        <v>3</v>
-      </c>
-      <c r="L4">
-        <v>1</v>
-      </c>
       <c r="M4">
         <v>1</v>
       </c>
@@ -13410,40 +13410,40 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C5">
+        <v>5</v>
+      </c>
+      <c r="D5">
+        <v>6</v>
+      </c>
+      <c r="E5">
+        <v>5</v>
+      </c>
+      <c r="F5">
+        <v>6</v>
+      </c>
+      <c r="G5">
+        <v>4</v>
+      </c>
+      <c r="H5">
+        <v>12</v>
+      </c>
+      <c r="I5">
         <v>7</v>
       </c>
-      <c r="D5">
-        <v>11</v>
-      </c>
-      <c r="E5">
-        <v>21</v>
-      </c>
-      <c r="F5">
-        <v>25</v>
-      </c>
-      <c r="G5">
-        <v>15</v>
-      </c>
-      <c r="H5">
-        <v>10</v>
-      </c>
-      <c r="I5">
-        <v>9</v>
-      </c>
       <c r="J5">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="K5">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="L5">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="M5">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -13451,40 +13451,40 @@
         <v>6</v>
       </c>
       <c r="B6">
+        <v>4</v>
+      </c>
+      <c r="C6">
+        <v>6</v>
+      </c>
+      <c r="D6">
+        <v>9</v>
+      </c>
+      <c r="E6">
+        <v>6</v>
+      </c>
+      <c r="F6">
         <v>10</v>
       </c>
-      <c r="C6">
+      <c r="G6">
+        <v>11</v>
+      </c>
+      <c r="H6">
+        <v>13</v>
+      </c>
+      <c r="I6">
+        <v>12</v>
+      </c>
+      <c r="J6">
         <v>10</v>
       </c>
-      <c r="D6">
-        <v>14</v>
-      </c>
-      <c r="E6">
-        <v>23</v>
-      </c>
-      <c r="F6">
-        <v>28</v>
-      </c>
-      <c r="G6">
-        <v>16</v>
-      </c>
-      <c r="H6">
-        <v>14</v>
-      </c>
-      <c r="I6">
-        <v>17</v>
-      </c>
-      <c r="J6">
-        <v>16</v>
-      </c>
       <c r="K6">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="L6">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="M6">
-        <v>13</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -15325,7 +15325,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23.7109375" customWidth="1"/>
@@ -15388,41 +15388,32 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2">
-        <v>4</v>
-      </c>
       <c r="C2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D2">
-        <v>3</v>
-      </c>
-      <c r="E2">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F2">
-        <v>9</v>
-      </c>
-      <c r="G2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H2">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I2">
         <v>4</v>
       </c>
       <c r="J2">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="K2">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M2">
-        <v>9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -15432,38 +15423,35 @@
       <c r="B3">
         <v>4</v>
       </c>
-      <c r="C3">
-        <v>5</v>
-      </c>
       <c r="D3">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E3">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F3">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="G3">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="H3">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="I3">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J3">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="K3">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="L3">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="M3">
-        <v>10</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -15473,17 +15461,14 @@
       <c r="B4">
         <v>1</v>
       </c>
-      <c r="D4">
-        <v>1</v>
-      </c>
-      <c r="E4">
-        <v>1</v>
-      </c>
-      <c r="J4">
-        <v>3</v>
+      <c r="H4">
+        <v>2</v>
       </c>
       <c r="K4">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="L4">
+        <v>1</v>
       </c>
       <c r="M4">
         <v>1</v>
@@ -15491,92 +15476,84 @@
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="B5">
+        <v>5</v>
+      </c>
+      <c r="C5">
+        <v>7</v>
+      </c>
+      <c r="D5">
+        <v>11</v>
+      </c>
+      <c r="E5">
+        <v>21</v>
+      </c>
+      <c r="F5">
+        <v>25</v>
+      </c>
+      <c r="G5">
+        <v>15</v>
+      </c>
+      <c r="H5">
+        <v>10</v>
+      </c>
+      <c r="I5">
+        <v>9</v>
+      </c>
+      <c r="J5">
+        <v>11</v>
       </c>
       <c r="K5">
-        <v>1</v>
+        <v>18</v>
+      </c>
+      <c r="L5">
+        <v>11</v>
+      </c>
+      <c r="M5">
+        <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B6">
+        <v>10</v>
+      </c>
+      <c r="C6">
+        <v>10</v>
+      </c>
+      <c r="D6">
+        <v>14</v>
+      </c>
+      <c r="E6">
         <v>23</v>
       </c>
-      <c r="C6">
+      <c r="F6">
+        <v>28</v>
+      </c>
+      <c r="G6">
+        <v>16</v>
+      </c>
+      <c r="H6">
+        <v>14</v>
+      </c>
+      <c r="I6">
+        <v>17</v>
+      </c>
+      <c r="J6">
+        <v>16</v>
+      </c>
+      <c r="K6">
         <v>31</v>
       </c>
-      <c r="D6">
+      <c r="L6">
         <v>22</v>
       </c>
-      <c r="E6">
-        <v>44</v>
-      </c>
-      <c r="F6">
-        <v>38</v>
-      </c>
-      <c r="G6">
-        <v>24</v>
-      </c>
-      <c r="H6">
-        <v>50</v>
-      </c>
-      <c r="I6">
-        <v>34</v>
-      </c>
-      <c r="J6">
-        <v>26</v>
-      </c>
-      <c r="K6">
-        <v>24</v>
-      </c>
-      <c r="L6">
-        <v>14</v>
-      </c>
       <c r="M6">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
-      <c r="A7" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B7">
-        <v>32</v>
-      </c>
-      <c r="C7">
-        <v>40</v>
-      </c>
-      <c r="D7">
-        <v>32</v>
-      </c>
-      <c r="E7">
-        <v>57</v>
-      </c>
-      <c r="F7">
-        <v>53</v>
-      </c>
-      <c r="G7">
-        <v>34</v>
-      </c>
-      <c r="H7">
-        <v>63</v>
-      </c>
-      <c r="I7">
-        <v>44</v>
-      </c>
-      <c r="J7">
-        <v>47</v>
-      </c>
-      <c r="K7">
-        <v>46</v>
-      </c>
-      <c r="L7">
-        <v>33</v>
-      </c>
-      <c r="M7">
-        <v>34</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -17357,10 +17334,10 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="18.7109375" customWidth="1"/>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
     <col min="2" max="2" width="4.7109375" customWidth="1"/>
     <col min="3" max="3" width="4.7109375" customWidth="1"/>
     <col min="4" max="4" width="4.7109375" customWidth="1"/>
@@ -17372,9 +17349,10 @@
     <col min="10" max="10" width="4.7109375" customWidth="1"/>
     <col min="11" max="11" width="4.7109375" customWidth="1"/>
     <col min="12" max="12" width="4.7109375" customWidth="1"/>
+    <col min="13" max="13" width="4.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12">
+    <row r="1" spans="1:13">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -17397,132 +17375,217 @@
         <v>2020</v>
       </c>
       <c r="H1" s="1">
+        <v>2021</v>
+      </c>
+      <c r="I1" s="1">
         <v>2022</v>
       </c>
-      <c r="I1" s="1">
+      <c r="J1" s="1">
         <v>2023</v>
       </c>
-      <c r="J1" s="1">
+      <c r="K1" s="1">
         <v>2024</v>
       </c>
-      <c r="K1" s="1">
+      <c r="L1" s="1">
         <v>2025</v>
       </c>
-      <c r="L1" s="1">
+      <c r="M1" s="1">
         <v>2026</v>
       </c>
     </row>
-    <row r="2" spans="1:12">
+    <row r="2" spans="1:13">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E2">
-        <v>2</v>
+        <v>5</v>
+      </c>
+      <c r="F2">
+        <v>9</v>
       </c>
       <c r="G2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H2">
-        <v>1</v>
+        <v>5</v>
+      </c>
+      <c r="I2">
+        <v>4</v>
+      </c>
+      <c r="J2">
+        <v>8</v>
       </c>
       <c r="K2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12">
+        <v>7</v>
+      </c>
+      <c r="L2">
+        <v>5</v>
+      </c>
+      <c r="M2">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B3">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C3">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D3">
-        <v>1</v>
+        <v>6</v>
+      </c>
+      <c r="E3">
+        <v>7</v>
+      </c>
+      <c r="F3">
+        <v>6</v>
+      </c>
+      <c r="G3">
+        <v>7</v>
+      </c>
+      <c r="H3">
+        <v>8</v>
       </c>
       <c r="I3">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="J3">
-        <v>1</v>
+        <v>10</v>
+      </c>
+      <c r="K3">
+        <v>12</v>
       </c>
       <c r="L3">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12">
+        <v>14</v>
+      </c>
+      <c r="M3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B4">
         <v>1</v>
       </c>
-      <c r="C4">
-        <v>8</v>
-      </c>
       <c r="D4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E4">
-        <v>7</v>
-      </c>
-      <c r="F4">
-        <v>4</v>
-      </c>
-      <c r="G4">
-        <v>4</v>
-      </c>
-      <c r="H4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12">
+        <v>1</v>
+      </c>
+      <c r="J4">
+        <v>3</v>
+      </c>
+      <c r="K4">
+        <v>2</v>
+      </c>
+      <c r="M4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5">
-        <v>5</v>
-      </c>
-      <c r="C5">
-        <v>11</v>
-      </c>
-      <c r="D5">
-        <v>5</v>
-      </c>
-      <c r="E5">
-        <v>9</v>
-      </c>
-      <c r="F5">
-        <v>4</v>
-      </c>
-      <c r="G5">
-        <v>5</v>
-      </c>
-      <c r="H5">
-        <v>2</v>
-      </c>
-      <c r="I5">
-        <v>1</v>
-      </c>
-      <c r="J5">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K5">
         <v>1</v>
       </c>
-      <c r="L5">
-        <v>2</v>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>23</v>
+      </c>
+      <c r="C6">
+        <v>31</v>
+      </c>
+      <c r="D6">
+        <v>22</v>
+      </c>
+      <c r="E6">
+        <v>44</v>
+      </c>
+      <c r="F6">
+        <v>38</v>
+      </c>
+      <c r="G6">
+        <v>24</v>
+      </c>
+      <c r="H6">
+        <v>50</v>
+      </c>
+      <c r="I6">
+        <v>34</v>
+      </c>
+      <c r="J6">
+        <v>26</v>
+      </c>
+      <c r="K6">
+        <v>24</v>
+      </c>
+      <c r="L6">
+        <v>14</v>
+      </c>
+      <c r="M6">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>32</v>
+      </c>
+      <c r="C7">
+        <v>40</v>
+      </c>
+      <c r="D7">
+        <v>32</v>
+      </c>
+      <c r="E7">
+        <v>57</v>
+      </c>
+      <c r="F7">
+        <v>53</v>
+      </c>
+      <c r="G7">
+        <v>34</v>
+      </c>
+      <c r="H7">
+        <v>63</v>
+      </c>
+      <c r="I7">
+        <v>44</v>
+      </c>
+      <c r="J7">
+        <v>47</v>
+      </c>
+      <c r="K7">
+        <v>46</v>
+      </c>
+      <c r="L7">
+        <v>33</v>
+      </c>
+      <c r="M7">
+        <v>34</v>
       </c>
     </row>
   </sheetData>
@@ -19070,10 +19133,10 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="1" max="1" width="18.7109375" customWidth="1"/>
     <col min="2" max="2" width="4.7109375" customWidth="1"/>
     <col min="3" max="3" width="4.7109375" customWidth="1"/>
     <col min="4" max="4" width="4.7109375" customWidth="1"/>
@@ -19085,10 +19148,9 @@
     <col min="10" max="10" width="4.7109375" customWidth="1"/>
     <col min="11" max="11" width="4.7109375" customWidth="1"/>
     <col min="12" max="12" width="4.7109375" customWidth="1"/>
-    <col min="13" max="13" width="4.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -19111,28 +19173,28 @@
         <v>2020</v>
       </c>
       <c r="H1" s="1">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="I1" s="1">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="J1" s="1">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="K1" s="1">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L1" s="1">
-        <v>2025</v>
-      </c>
-      <c r="M1" s="1">
         <v>2026</v>
       </c>
     </row>
-    <row r="2" spans="1:13">
+    <row r="2" spans="1:12">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="B2">
+        <v>2</v>
+      </c>
       <c r="C2">
         <v>1</v>
       </c>
@@ -19140,22 +19202,19 @@
         <v>1</v>
       </c>
       <c r="E2">
-        <v>1</v>
-      </c>
-      <c r="F2">
-        <v>1</v>
-      </c>
-      <c r="J2">
+        <v>2</v>
+      </c>
+      <c r="G2">
+        <v>1</v>
+      </c>
+      <c r="H2">
         <v>1</v>
       </c>
       <c r="K2">
-        <v>6</v>
-      </c>
-      <c r="L2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
@@ -19168,124 +19227,78 @@
       <c r="D3">
         <v>1</v>
       </c>
-      <c r="E3">
-        <v>3</v>
-      </c>
-      <c r="H3">
-        <v>1</v>
-      </c>
       <c r="I3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J3">
         <v>1</v>
       </c>
-      <c r="K3">
-        <v>3</v>
-      </c>
       <c r="L3">
         <v>2</v>
       </c>
-      <c r="M3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
+    </row>
+    <row r="4" spans="1:12">
       <c r="A4" s="1" t="s">
-        <v>3</v>
+        <v>5</v>
+      </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="C4">
+        <v>8</v>
       </c>
       <c r="D4">
-        <v>1</v>
-      </c>
-      <c r="L4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
+        <v>3</v>
+      </c>
+      <c r="E4">
+        <v>7</v>
+      </c>
+      <c r="F4">
+        <v>4</v>
+      </c>
+      <c r="G4">
+        <v>4</v>
+      </c>
+      <c r="H4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12">
       <c r="A5" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5">
+        <v>5</v>
+      </c>
+      <c r="C5">
+        <v>11</v>
+      </c>
+      <c r="D5">
+        <v>5</v>
+      </c>
+      <c r="E5">
+        <v>9</v>
+      </c>
+      <c r="F5">
         <v>4</v>
       </c>
       <c r="G5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
-      <c r="A6" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B6">
-        <v>4</v>
-      </c>
-      <c r="C6">
-        <v>2</v>
-      </c>
-      <c r="D6">
-        <v>8</v>
-      </c>
-      <c r="E6">
-        <v>5</v>
-      </c>
-      <c r="F6">
-        <v>4</v>
-      </c>
-      <c r="G6">
-        <v>4</v>
-      </c>
-      <c r="I6">
-        <v>3</v>
-      </c>
-      <c r="J6">
-        <v>4</v>
-      </c>
-      <c r="K6">
-        <v>6</v>
-      </c>
-      <c r="L6">
-        <v>5</v>
-      </c>
-      <c r="M6">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
-      <c r="A7" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B7">
-        <v>6</v>
-      </c>
-      <c r="C7">
-        <v>5</v>
-      </c>
-      <c r="D7">
-        <v>11</v>
-      </c>
-      <c r="E7">
-        <v>9</v>
-      </c>
-      <c r="F7">
-        <v>5</v>
-      </c>
-      <c r="G7">
-        <v>5</v>
-      </c>
-      <c r="H7">
-        <v>1</v>
-      </c>
-      <c r="I7">
-        <v>5</v>
-      </c>
-      <c r="J7">
-        <v>6</v>
-      </c>
-      <c r="K7">
-        <v>15</v>
-      </c>
-      <c r="L7">
-        <v>13</v>
-      </c>
-      <c r="M7">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="H5">
+        <v>2</v>
+      </c>
+      <c r="I5">
+        <v>1</v>
+      </c>
+      <c r="J5">
+        <v>1</v>
+      </c>
+      <c r="K5">
+        <v>1</v>
+      </c>
+      <c r="L5">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -20311,10 +20324,10 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="18.7109375" customWidth="1"/>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
     <col min="2" max="2" width="4.7109375" customWidth="1"/>
     <col min="3" max="3" width="4.7109375" customWidth="1"/>
     <col min="4" max="4" width="4.7109375" customWidth="1"/>
@@ -20386,26 +20399,14 @@
       <c r="F2">
         <v>1</v>
       </c>
-      <c r="G2">
-        <v>4</v>
-      </c>
-      <c r="H2">
-        <v>1</v>
-      </c>
-      <c r="I2">
-        <v>1</v>
-      </c>
       <c r="J2">
         <v>1</v>
       </c>
       <c r="K2">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L2">
-        <v>2</v>
-      </c>
-      <c r="M2">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -20416,127 +20417,129 @@
         <v>2</v>
       </c>
       <c r="C3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D3">
         <v>1</v>
       </c>
       <c r="E3">
-        <v>2</v>
-      </c>
-      <c r="F3">
-        <v>2</v>
-      </c>
-      <c r="G3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H3">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I3">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J3">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="K3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L3">
         <v>2</v>
       </c>
       <c r="M3">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="K4">
+        <v>3</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="L4">
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5">
-        <v>6</v>
-      </c>
-      <c r="C5">
-        <v>8</v>
-      </c>
-      <c r="D5">
-        <v>6</v>
-      </c>
-      <c r="E5">
-        <v>7</v>
-      </c>
-      <c r="F5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G5">
-        <v>5</v>
-      </c>
-      <c r="H5">
-        <v>1</v>
-      </c>
-      <c r="I5">
-        <v>7</v>
-      </c>
-      <c r="J5">
-        <v>11</v>
-      </c>
-      <c r="K5">
-        <v>8</v>
-      </c>
-      <c r="L5">
-        <v>5</v>
-      </c>
-      <c r="M5">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B6">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C6">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="D6">
         <v>8</v>
       </c>
       <c r="E6">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="F6">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G6">
+        <v>4</v>
+      </c>
+      <c r="I6">
+        <v>3</v>
+      </c>
+      <c r="J6">
+        <v>4</v>
+      </c>
+      <c r="K6">
+        <v>6</v>
+      </c>
+      <c r="L6">
+        <v>5</v>
+      </c>
+      <c r="M6">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>6</v>
+      </c>
+      <c r="C7">
+        <v>5</v>
+      </c>
+      <c r="D7">
         <v>11</v>
       </c>
-      <c r="H6">
-        <v>6</v>
-      </c>
-      <c r="I6">
+      <c r="E7">
+        <v>9</v>
+      </c>
+      <c r="F7">
+        <v>5</v>
+      </c>
+      <c r="G7">
+        <v>5</v>
+      </c>
+      <c r="H7">
+        <v>1</v>
+      </c>
+      <c r="I7">
+        <v>5</v>
+      </c>
+      <c r="J7">
+        <v>6</v>
+      </c>
+      <c r="K7">
+        <v>15</v>
+      </c>
+      <c r="L7">
         <v>13</v>
       </c>
-      <c r="J6">
-        <v>19</v>
-      </c>
-      <c r="K6">
-        <v>15</v>
-      </c>
-      <c r="L6">
-        <v>9</v>
-      </c>
-      <c r="M6">
-        <v>9</v>
+      <c r="M7">
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>